<commit_message>
Fix BUG-038: Terms of Service always displayed in English
SECTIONS array was at module scope — t() called once on load, ignoring
language changes. Moved inside component; all strings use titleKey/bodyKey
refs + t() with TranslationKey cast. Added 22 i18n keys (EN + HE) for
all 10 ToS sections, intro, and last-updated subtitle.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H81"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -1856,9 +1856,425 @@
         <v>done</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B66" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C66" t="str">
+        <v>src/integrations/supabase/client.ts, src/integrations/payment/payme.ts, src/integrations/ai/claudeClient.ts</v>
+      </c>
+      <c r="D66" t="str">
+        <v>BUG-030: Add eslint-disable-next-line no-unused-vars to stub parameters (_userId, _req) in integration files to fix lint errors</v>
+      </c>
+      <c r="E66" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F66" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Agent 5</v>
+      </c>
+      <c r="H66" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B67" t="str">
+        <v>10:30</v>
+      </c>
+      <c r="C67" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D67" t="str">
+        <v>BUG-031: Language toggle indicator invisible when Hebrew selected. Moved width/borderRadius from Tailwind arbitrary-value class (w-[calc(50%-4px)]) to inline style — Tailwind stripped the spaces in calc() generating invalid CSS</v>
+      </c>
+      <c r="E67" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F67" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H67" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B68" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C68" t="str">
+        <v>src/components/WhatsAppButton.tsx</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Add automatic image copy to clipboard on WhatsApp button click; Hebrew popup with paste instructions; close button; stores image as base64 canvas snapshot</v>
+      </c>
+      <c r="E68" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F68" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H68" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B69" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C69" t="str">
+        <v>src/services/communicationService.ts</v>
+      </c>
+      <c r="D69" t="str">
+        <v>BUG-032/033/034: Fix double 00-prefix in WhatsApp URL builder; add guard for empty phone string; remove deprecated execCommand clipboard fallback</v>
+      </c>
+      <c r="E69" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F69" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H69" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B70" t="str">
+        <v>11:30</v>
+      </c>
+      <c r="C70" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Add @hebcal/core Hebrew date (gematria) to every calendar cell; Rosh Chodesh shows month name; Hebrew month names in pill badge</v>
+      </c>
+      <c r="E70" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F70" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H70" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B71" t="str">
+        <v>11:30</v>
+      </c>
+      <c r="C71" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Add 3 i18n keys: whatsapp_image_ready_title, whatsapp_image_paste_hint, whatsapp_image_paste_steps (EN + HE)</v>
+      </c>
+      <c r="E71" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F71" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Foundation-Agent</v>
+      </c>
+      <c r="H71" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B72" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C72" t="str">
+        <v>AGENTS.md</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Create AGENTS.md — documentation of all 8 agent definitions, roles, and iteration action logs</v>
+      </c>
+      <c r="E72" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F72" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H72" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B73" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C73" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Add 20 i18n keys: urgency_critical/high/medium/low, go_back, action_wish_birthday_today/days, action_wish_holiday_days, action_reconnect_days, action_checkin, action_followup, holiday_major, holiday_moreContacts (EN + HE)</v>
+      </c>
+      <c r="E73" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F73" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Foundation-Agent</v>
+      </c>
+      <c r="H73" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B74" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C74" t="str">
+        <v>src/core/scoringSystem.ts</v>
+      </c>
+      <c r="D74" t="str">
+        <v>BUG-020: Fix getBirthdayDaysUntil using date-fns differenceInCalendarDays — prevents wrong result on DST change days</v>
+      </c>
+      <c r="E74" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F74" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H74" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B75" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C75" t="str">
+        <v>src/components/Navigation.tsx, src/screens/ContactDetailScreen.tsx, src/screens/HolidayDetailScreen.tsx, src/screens/DashboardScreen.tsx, src/screens/GroupsScreen.tsx, src/components/ui/Modal.tsx, src/screens/premium/ImportContactsScreen.tsx, src/components/ContactCard.tsx, src/index.css</v>
+      </c>
+      <c r="D75" t="str">
+        <v>BUG-036 / FINDINGS 25A/20/23/28A/30B/60/66/67/69: aria-labels localized, urgency/frequency labels translated, group+dashboard cards converted to &lt;button&gt;, .btn:focus-visible ring added, setImporting in finally, decorative icon aria-hidden</v>
+      </c>
+      <c r="E75" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F75" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H75" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B76" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C76" t="str">
+        <v>src/screens/SettingsScreen.tsx, src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D76" t="str">
+        <v>SECURITY: Wrap Danger Zone section and demo premium activation button in import.meta.env.DEV — both are completely tree-shaken from production builds by rolldown</v>
+      </c>
+      <c r="E76" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F76" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H76" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B77" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C77" t="str">
+        <v>src/utils/hebrewDateUtils.ts</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Create hebrewDateUtils.ts — getHebrewDateStr(isoDate) converts Gregorian ISO date to Hebrew gematria string (e.g. ד׳ באייר תשפ״ו); uses local-time Date construction to avoid UTC timezone shifts</v>
+      </c>
+      <c r="E77" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F77" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H77" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B78" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C78" t="str">
+        <v>src/data/holidays.ts</v>
+      </c>
+      <c r="D78" t="str">
+        <v>BUG-037: Yom HaAtzmaut 2026 was hardcoded as 2026-04-29 (wrong by 8 days); replaced with runtime computation via HebrewCalendar.getHolidaysForYearArray(5786, true) from @hebcal/core; correct date is 2026-04-21 (ד׳ באייר תשפ״ו)</v>
+      </c>
+      <c r="E78" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F78" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H78" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B79" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C79" t="str">
+        <v>src/components/HolidayCard.tsx, src/screens/HolidayDetailScreen.tsx</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Add Hebrew date badge (gematria format) to HolidayCard compact/full views and HolidayDetailScreen hero banner for all dateType === "hebrew" holidays</v>
+      </c>
+      <c r="E79" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F79" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H79" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B80" t="str">
+        <v>17:00</v>
+      </c>
+      <c r="C80" t="str">
+        <v>src/screens/TermsScreen.tsx</v>
+      </c>
+      <c r="D80" t="str">
+        <v>BUG-038: Terms of Service page always showed English. Root cause: SECTIONS array was at module scope — t() calls were made once on load, ignoring language changes. Fix: moved SECTIONS inside component; replaced all hardcoded strings with titleKey/bodyKey references + t() calls with as const + TranslationKey cast</v>
+      </c>
+      <c r="E80" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F80" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G80" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H80" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B81" t="str">
+        <v>17:00</v>
+      </c>
+      <c r="C81" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Add 22 i18n keys for Terms of Service: terms_lastUpdated, terms_intro, terms_s1_title/body through terms_s10_title/body — full Hebrew translations for all 10 sections (EN + HE)</v>
+      </c>
+      <c r="E81" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F81" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Foundation-Agent</v>
+      </c>
+      <c r="H81" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H81"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add local analytics foundation (no backend)
analyticsService: getAnonymousUserId() persists UUID to nm_user_id;
trackEvent() stores up to 100 events FIFO in nm_events. Tracks:
app_open, contact_created, greeting_sent (+ channel), contacts_imported
(+ count). Silent failure guarantees analytics never breaks the app.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H83"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2272,9 +2272,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B82" t="str">
+        <v>18:00</v>
+      </c>
+      <c r="C82" t="str">
+        <v>src/services/analyticsService.ts</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Create local analytics service: getAnonymousUserId() generates/persists UUID in localStorage (nm_user_id); trackEvent(name, metadata?) stores up to 100 events FIFO in nm_events. No backend, no dashboard, zero side effects.</v>
+      </c>
+      <c r="E82" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F82" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G82" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H82" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B83" t="str">
+        <v>18:00</v>
+      </c>
+      <c r="C83" t="str">
+        <v>src/App.tsx, src/screens/ContactFormScreen.tsx, src/components/ChannelPicker.tsx, src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Add trackEvent calls for 4 events: app_open (AppShell mount), contact_created (new contact only), greeting_sent (with channel metadata), contacts_imported (with count metadata)</v>
+      </c>
+      <c r="E83" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F83" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H83" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H83"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix BUG-039 (calendar birthdays) + add Hebrew birthday field
BUG-039: CalendarScreen now shows a pink dot for birthdays on cells;
birthday section panel lists contacts for selected day or full month.
birthdayMap useMemo handles hebrewBirthday (priority) and birthday fields.

FEATURE: Optional hebrewBirthday field on Contact ("DD-MM" format —
Hebrew day + month, year-agnostic). hebrewBirthdayToGregorianInCalendarYear()
converts to Gregorian. UI in ContactForm premium section (Judaism contacts);
day+month dropdowns + clear button. 7 new i18n keys (EN + HE).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H88"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2324,9 +2324,139 @@
         <v>done</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B84" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="C84" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D84" t="str">
+        <v>BUG-039: Contact birthdays never appeared in calendar. Added birthdayMap useMemo — builds Map&lt;date-string, Contact[]&gt; for visible month using hebrewBirthday (priority) or birthday. Pink dot (#EC4899) added to cell dots row. Birthday panel section added below calendar showing contact name cards for selected day / full month.</v>
+      </c>
+      <c r="E84" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F84" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H84" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B85" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="C85" t="str">
+        <v>src/types/index.ts</v>
+      </c>
+      <c r="D85" t="str">
+        <v>FEATURE: Add optional hebrewBirthday?: string field to Contact interface — stored as "DD-MM" (Hebrew day-month, year-agnostic). Additive only; does not affect existing birthday field.</v>
+      </c>
+      <c r="E85" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F85" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G85" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H85" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B86" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="C86" t="str">
+        <v>src/utils/hebrewDateUtils.ts</v>
+      </c>
+      <c r="D86" t="str">
+        <v>FEATURE: Add hebrewBirthdayToGregorianInCalendarYear(hebrewBirthday, gregorianYear) — converts "DD-MM" Hebrew date to Gregorian Date for a given year; tries approxHYear and approxHYear+1 to handle year boundary; returns null for invalid combos (e.g. Adar II in non-leap year)</v>
+      </c>
+      <c r="E86" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F86" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G86" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H86" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B87" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="C87" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D87" t="str">
+        <v>FEATURE: Add Hebrew Birthday UI in premium section — shown for Judaism contacts or when hebrewBirthday already set. Two dropdowns (day 1–30, Hebrew month 1–12 with names). Derives day/month from form.hebrewBirthday via useMemo. Clear button removes the field. Saved as "DD-MM" string.</v>
+      </c>
+      <c r="E87" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F87" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G87" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H87" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B88" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="C88" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Add 7 i18n keys (EN + HE): calendar_birthdays, calendar_birthdayLabel, calendar_birthdaysOn, contactForm_hebrewBirthday, contactForm_hebrewBirthdayDay, contactForm_hebrewBirthdayMonth, contactForm_hebrewBirthdayClear</v>
+      </c>
+      <c r="E88" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F88" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G88" t="str">
+        <v>Foundation-Agent</v>
+      </c>
+      <c r="H88" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H88"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 2 iter 17: i18n, accessibility, celebration feedback (BL-014–018, BL-041)
- BL-015: GreetingEditorScreen tier descs + signature placeholder via t(); 4 new i18n keys
- BL-016: ContactCard action labels translated via ACTION_KEY map + useT()
- BL-017/018: aria-label on Edit/Regenerate/Copy; aria-expanded on toggle buttons
- BL-041: Mark as Contacted celebration — 6-emoji particle burst, Web Audio ping, haptic vibrate(40); respects prefers-reduced-motion
- changelog.xlsx updated (92 entries); QA checklist updated (56/57 passing)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H93"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2454,9 +2454,139 @@
         <v>done</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B89" t="str">
+        <v>20:00</v>
+      </c>
+      <c r="C89" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D89" t="str">
+        <v>BL-015: Replace hardcoded tier desc strings with i18n keys (greeting_tier_*_desc). Signature placeholder via t('greeting_signature_placeholder'). BL-017: aria-label on Regenerate and Copy icon buttons. BL-018: aria-expanded on Advanced tone + Signature toggle buttons. aria-hidden on decorative icons.</v>
+      </c>
+      <c r="E89" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F89" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G89" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H89" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B90" t="str">
+        <v>20:00</v>
+      </c>
+      <c r="C90" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D90" t="str">
+        <v>BL-015: Add 4 i18n keys (EN + HE): greeting_tier_casual_desc, greeting_tier_professional_desc, greeting_tier_vip_desc, greeting_signature_placeholder</v>
+      </c>
+      <c r="E90" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F90" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G90" t="str">
+        <v>Foundation-Agent</v>
+      </c>
+      <c r="H90" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B91" t="str">
+        <v>20:00</v>
+      </c>
+      <c r="C91" t="str">
+        <v>src/components/ContactCard.tsx</v>
+      </c>
+      <c r="D91" t="str">
+        <v>BL-016: Add ACTION_KEY Record&lt;SuggestedActionType, TranslationKey&gt; map. Use useT() + t(ACTION_KEY[...]) to display action label in current language instead of raw English label string.</v>
+      </c>
+      <c r="E91" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F91" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G91" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H91" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B92" t="str">
+        <v>20:00</v>
+      </c>
+      <c r="C92" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D92" t="str">
+        <v>BL-017: aria-label on Edit icon button via t('contactForm_edit'). BL-041: Add celebration feedback on Mark as Contacted — 6 emoji particle burst (.animate-particle with --tx/--ty CSS vars), Web Audio oscillator ping (880→1200Hz ramp, 0.4s), haptic navigator.vibrate(40). Respects prefers-reduced-motion. useState celebrating moved before early return to comply with hooks rules.</v>
+      </c>
+      <c r="E92" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F92" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G92" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H92" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B93" t="str">
+        <v>20:00</v>
+      </c>
+      <c r="C93" t="str">
+        <v>src/index.css</v>
+      </c>
+      <c r="D93" t="str">
+        <v>BL-041: Add @keyframes particleBurst (translate + scale to 0 + opacity fade driven by --tx/--ty CSS custom properties) and .animate-particle utility class (1.2s ease-out forwards).</v>
+      </c>
+      <c r="E93" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F93" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G93" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H93" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H88"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H93"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix BUG-040: reconstruct missing iterations 13-17 in iteration_log.md
Iterations 13-17 (all 2026-04-28) were never appended to iteration_log.md.
Reconstructed from changelog_queue.json as the sole authoritative source.
Agent 2/3 columns marked TBD where research_notes/review_notes have no entries.
Log is now continuous 0-17. BUG_REPORT.md updated with BUG-040 entry.
changelog.xlsx at 94 entries.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H95"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2584,9 +2584,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B94" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C94" t="str">
+        <v>agent_state/iteration_log.md</v>
+      </c>
+      <c r="D94" t="str">
+        <v>BUG-040 fix: reconstructed iterations 13–17 from changelog_queue.json. All 5 entries appended: iter 13 (Hebrew date display + BUG-037), iter 14 (BUG-038 Terms fix), iter 15 (analytics foundation), iter 16 (BUG-039 birthday calendar + Hebrew birthday feature), iter 17 (BL-015/016/017/018/041 i18n + accessibility + celebration). Agent 2/3 columns marked TBD where source files have no entries. Log is now continuous 0–17.</v>
+      </c>
+      <c r="E94" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F94" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G94" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H94" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B95" t="str">
+        <v>20:30</v>
+      </c>
+      <c r="C95" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Added BUG-040 entry: iteration_log.md missing iterations 13–17. Marked fixed.</v>
+      </c>
+      <c r="E95" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F95" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H95" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H95"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 2 complete: React.lazy (BL-019) + scoringSystem cache (BL-020)
BL-019: 13 screens converted to lazy chunks via React.lazy; Suspense fallback
moved inside WithNav so BottomNav stays visible during navigation. Main bundle
reduced from 435 kB to 285 kB raw (-37 kB gzip). Premium route inner Suspense
wrappers removed — outer WithNav Suspense handles all lazy screens uniformly.

BL-020: Module-level Map cache in scoringSystem.ts keyed by `id|updatedAt`.
Eliminates redundant score calculations for unchanged contacts on every render.

BL-021/022: Confirmed already implemented — pull-to-refresh and no standalone
no-op refresh button. Sprint 2 backlog fully cleared.

changelog.xlsx at 96 entries; QA 56/57 passing.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H97"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2636,9 +2636,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B96" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="C96" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="D96" t="str">
+        <v>BL-019: Convert 13 screens to React.lazy (CalendarScreen, HolidayDetailScreen, ContactsScreen, ContactDetailScreen, ContactFormScreen, GreetingEditorScreen, GroupsScreen, SettingsScreen, UpgradeScreen, AboutScreen, PrivacyScreen, TermsScreen, WhatsNewScreen). Move Suspense fallback into WithNav so BottomNav stays visible during load. Remove now-redundant inner Suspense from 3 premium routes. Main bundle: 435 kB → 285 kB raw (-150 kB), 130 kB → 93 kB gzip (-37 kB).</v>
+      </c>
+      <c r="E96" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F96" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H96" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B97" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="C97" t="str">
+        <v>src/core/scoringSystem.ts</v>
+      </c>
+      <c r="D97" t="str">
+        <v>BL-020: Add module-level scoreCache Map&lt;string, RelationshipScore&gt; keyed by `contact.id|contact.updatedAt`. calculateRelationshipScore checks cache on entry and sets result before return. Eliminates redundant scoring for unchanged contacts on every render. Stale results impossible since updatedAt is always stamped on mutation.</v>
+      </c>
+      <c r="E97" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F97" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H97" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H97"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 3: celebrationType field, overdue notifications, device contacts import
BL-026: Add CelebrationType (Jewish/Christian/Muslim/Druze/Secular) to Contact
type; CELEBRATION_TO_RELIGION map in scoringSystem.ts for holiday filtering;
celebrationType Select in ContactForm Cultural section; 10 i18n keys EN+HE.

BL-023: Add overdue-contact notification (45-day threshold) to
notificationService.ts; skips contacts covered by birthday reminder (within 7d);
notif_overdue + notif_overdue_body keys in both locales.

BL-030: Install @capacitor-community/contacts; new DeviceContactsScreen with
full consent/permission/list/import flow, phone dedup, Capacitor.isNativePlatform()
web fallback; Premium-gated /device-contacts route; shortcut in ImportContactsScreen.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:H105"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2675,22 +2675,218 @@
       <c r="D97" t="str">
         <v>BL-020: Add module-level scoreCache Map&lt;string, RelationshipScore&gt; keyed by `contact.id|contact.updatedAt`. calculateRelationshipScore checks cache on entry and sets result before return. Eliminates redundant scoring for unchanged contacts on every render. Stale results impossible since updatedAt is always stamped on mutation.</v>
       </c>
-      <c r="E97" t="str">
-        <v>improvement</v>
-      </c>
-      <c r="F97" t="str">
-        <v>code_change</v>
-      </c>
-      <c r="G97" t="str">
-        <v>Agent 1</v>
-      </c>
-      <c r="H97" t="str">
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B98" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C98" t="str">
+        <v>src/types/index.ts</v>
+      </c>
+      <c r="D98" t="str">
+        <v>BL-026: Add CelebrationType union type (Jewish|Christian|Muslim|Druze|Secular); add optional celebrationType field to Contact interface</v>
+      </c>
+      <c r="E98" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F98" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Foundation Agent</v>
+      </c>
+      <c r="H98" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B99" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C99" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D99" t="str">
+        <v>BL-026+BL-023+BL-030: Add 34 i18n keys — celebrationType_* (5 values EN+HE), contactForm_celebrationType, notif_overdue/notif_overdue_body, 14 deviceContacts_* keys, premium_feat_device_contacts — all in EN and HE</v>
+      </c>
+      <c r="E99" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F99" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G99" t="str">
+        <v>Foundation Agent</v>
+      </c>
+      <c r="H99" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B100" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C100" t="str">
+        <v>src/core/scoringSystem.ts</v>
+      </c>
+      <c r="D100" t="str">
+        <v>BL-026: Add CELEBRATION_TO_RELIGION map; update getUpcomingHolidaysForContact to prefer celebrationType over religion when set, falling back to religion for existing contacts</v>
+      </c>
+      <c r="E100" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F100" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G100" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H100" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B101" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C101" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D101" t="str">
+        <v>BL-026: Add celebrationType Select dropdown to Cultural &amp; Language section; wire into form state and handleSave; import CelebrationType type</v>
+      </c>
+      <c r="E101" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F101" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G101" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H101" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B102" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C102" t="str">
+        <v>src/services/notificationService.ts</v>
+      </c>
+      <c r="D102" t="str">
+        <v>BL-023: Add overdue-contact reminder — fires when daysSince &gt;= 45 days with no upcoming birthday within 7 days; dedup via existing nm_notif_sent localStorage mechanism</v>
+      </c>
+      <c r="E102" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F102" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G102" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H102" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B103" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C103" t="str">
+        <v>src/screens/DeviceContactsScreen.tsx</v>
+      </c>
+      <c r="D103" t="str">
+        <v>BL-030: New screen — consent → permission request → device contact list with checkboxes → import with phone dedup. Capacitor.isNativePlatform() guard shows graceful web-only message. Imports @capacitor-community/contacts. Premium-gated via App.tsx route.</v>
+      </c>
+      <c r="E103" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F103" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G103" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H103" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B104" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C104" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="D104" t="str">
+        <v>BL-030: Add DeviceContactsScreen lazy import; add route /device-contacts with Premium gate (isPremium ? DeviceContactsScreen : UpgradeScreen)</v>
+      </c>
+      <c r="E104" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F104" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H104" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B105" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C105" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D105" t="str">
+        <v>BL-030: Add "Import from Phone" shortcut card at top of Import screen; navigates to /device-contacts</v>
+      </c>
+      <c r="E105" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F105" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G105" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H105" t="str">
         <v>done</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H105"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix BUG-043/044: multi-day holiday calendar dots + Sukkot 2026
BUG-043: CalendarScreen getHolidaysForDay previously matched only the
start date via isSameDay. Now uses numeric YYYYMMDD range comparison
so every day of Sukkot, Hanukkah, Passover, etc. shows a dot in the
calendar grid. Monthly list filter updated to include holidays that
overlap the visible month, not just those that start in it.

BUG-044: Add missing sukkot-2026 entry (2026-09-25 to 2026-10-02,
15–22 Tishrei 5787), covering Hoshana Rabbah and Shemini Atzeret /
Simchat Torah. Matches existing sukkot-2025 pattern.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H107"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2884,9 +2884,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B106" t="str">
+        <v>23:00</v>
+      </c>
+      <c r="C106" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D106" t="str">
+        <v>BUG-043: Fix multi-day holidays only showing dot on first day. Replace isSameDay check with numeric YYYYMMDD range [startNum, endNum] in getHolidaysForDay. Fix monthly list to show holidays overlapping the visible month (not just holidays that start in the month). Remove unused isSameMonth import.</v>
+      </c>
+      <c r="E106" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F106" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G106" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H106" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B107" t="str">
+        <v>23:00</v>
+      </c>
+      <c r="C107" t="str">
+        <v>src/data/holidays.ts</v>
+      </c>
+      <c r="D107" t="str">
+        <v>BUG-044: Add missing sukkot-2026 entry (Sep 25 – Oct 2, 2026 / 15–22 Tishrei 5787). Covers full festival including Hoshana Rabbah and Shemini Atzeret / Simchat Torah. Matches existing sukkot-2025 pattern.</v>
+      </c>
+      <c r="E107" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F107" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G107" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H107" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H107"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BL-045: Improve celebration feedback on Mark as Contacted
Sound: Replace harsh 880→1200Hz oscillator with a pleasant C5/E5/G5
major triad arpeggio — three staggered sine waves decaying over ~0.75s.

Animation: 10 particles (was 6), text-xl size, wider spread ±85px
horizontal / ±110px vertical. New scale-pop keyframe (0.4 → 1.6 → 0)
gives a visible "pop then fly" effect vs previous translate-only.
Duration 1.4s. prefers-reduced-motion guard unchanged.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H109"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2936,9 +2936,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B108" t="str">
+        <v>23:30</v>
+      </c>
+      <c r="C108" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D108" t="str">
+        <v>BL-045: Replace harsh oscillator with C5/E5/G5 major triad arpeggio (3 sine waves, ~0.75s, pleasant chord). Expand particles from 6 to 10, size text-xl (was text-base), wider spread ±85px h / ±110px v. Animation delay stagger 50ms per particle (was 40ms). State clear timeout 1600ms.</v>
+      </c>
+      <c r="E108" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F108" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H108" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B109" t="str">
+        <v>23:30</v>
+      </c>
+      <c r="C109" t="str">
+        <v>src/index.css</v>
+      </c>
+      <c r="D109" t="str">
+        <v>BL-045: Update particleBurst keyframe — scale-pop effect: 0.4 → 1.6 → 0 across 0/18%/100% keyframe stops, giving a visible "pop then fly" motion. Animation class duration 1.2s → 1.4s.</v>
+      </c>
+      <c r="E109" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F109" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G109" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H109" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H109"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 4: Export to CSV (BL-025) + WCAG 2.5.5 tap targets (BL-029)
BL-025: New exportService.ts with PapaParse CSV export including UTF-8 BOM for Hebrew Excel compatibility. Export button added to Settings > Premium Features with 2.5s success feedback.

BL-029: 9 icon-only buttons upgraded to min-48×48px tap targets across Navigation, Modal, ContactDetail, ContactForm, GroupsScreen, GreetingEditor, HolidayDetail, and BirthdayGreetingEditor.

Build: clean (2151 modules). Lint: clean. QA: 56/57 ✅.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H120"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -2988,9 +2988,295 @@
         <v>done</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B110" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C110" t="str">
+        <v>src/services/exportService.ts</v>
+      </c>
+      <c r="D110" t="str">
+        <v>BL-025 (Sprint 4): New exportContactsToCSV() using PapaParse. Exports all Contact fields to CSV with UTF-8 BOM for Hebrew Excel compatibility. Downloads as nevermiss-contacts-YYYY-MM-DD.csv.</v>
+      </c>
+      <c r="E110" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F110" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G110" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H110" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B111" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C111" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D111" t="str">
+        <v>BL-025 (Sprint 4): Added Export Contacts to CSV button in Premium Features card. exportDone state shows success feedback for 2.5s.</v>
+      </c>
+      <c r="E111" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F111" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G111" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H111" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B112" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C112" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D112" t="str">
+        <v>BL-025 (Sprint 4): Added i18n keys settings_exportContacts + settings_exportSuccess in EN+HE.</v>
+      </c>
+      <c r="E112" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F112" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G112" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H112" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B113" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C113" t="str">
+        <v>src/components/Navigation.tsx</v>
+      </c>
+      <c r="D113" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Back button in PageHeader changed to min-w/h-[48px] flex items-center justify-center — 48×48px minimum tap target.</v>
+      </c>
+      <c r="E113" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F113" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H113" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B114" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C114" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D114" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Delete icon button in ContactForm PageHeader changed to min-w/h-[48px] tap target.</v>
+      </c>
+      <c r="E114" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F114" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G114" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H114" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B115" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C115" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D115" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Edit and Delete icon buttons on group cards changed to min-w/h-[48px] tap targets.</v>
+      </c>
+      <c r="E115" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F115" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H115" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B116" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C116" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D116" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Regenerate and Copy icon buttons changed to min-w/h-[48px] tap targets.</v>
+      </c>
+      <c r="E116" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F116" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G116" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H116" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B117" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C117" t="str">
+        <v>src/components/ui/Modal.tsx</v>
+      </c>
+      <c r="D117" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Close (X) button in Modal header changed to min-w/h-[48px] tap target.</v>
+      </c>
+      <c r="E117" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F117" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G117" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H117" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B118" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C118" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D118" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Edit icon button in ContactDetail PageHeader changed to min-w/h-[48px] tap target.</v>
+      </c>
+      <c r="E118" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F118" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G118" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H118" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B119" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C119" t="str">
+        <v>src/screens/HolidayDetailScreen.tsx</v>
+      </c>
+      <c r="D119" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Copy greeting icon button changed to min-w/h-[48px] tap target.</v>
+      </c>
+      <c r="E119" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F119" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G119" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H119" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B120" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C120" t="str">
+        <v>src/screens/premium/BirthdayGreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D120" t="str">
+        <v>BL-029 (Sprint 4) WCAG 2.5.5: Regenerate and Copy icon buttons in BirthdayGreetingEditor changed to min-w/h-[48px] tap targets.</v>
+      </c>
+      <c r="E120" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F120" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G120" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H120" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H120"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 4: Haptic feedback (BL-024), Backup/restore (BL-034), Duplicate detection (BL-035)
BL-024: hapticService.ts with Capacitor.isNativePlatform() guard, wired to contact save, greeting send, and coupon redemption. No-op in browser.

BL-034: exportBackupJSON/importBackupJSON in storageService; Backup + Restore buttons in Settings Premium Features card with success/error feedback.

BL-035: findDuplicate() checks exact name + phone (7+ digits) on new contacts; Modal warns user with existing contact name, offers Save Anyway or Cancel.

Build: clean (2155 modules). Lint: clean. QA: 56/57 ✅. Changelog: 125 entries.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H126"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -3274,9 +3274,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B121" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C121" t="str">
+        <v>src/services/hapticService.ts</v>
+      </c>
+      <c r="D121" t="str">
+        <v>BL-024 (Sprint 4): New hapticService with hapticLight/Medium/Success/Error. Uses Capacitor.isNativePlatform() guard — graceful no-op in browser. ImpactStyle.Light/Medium and NotificationType.Success/Error.</v>
+      </c>
+      <c r="E121" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F121" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G121" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H121" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B122" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C122" t="str">
+        <v>src/screens/ContactFormScreen.tsx + src/components/ChannelPicker.tsx + src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D122" t="str">
+        <v>BL-024 (Sprint 4): Haptic wired to 3 key actions — hapticSuccess after contact save, hapticMedium on greeting channel select, hapticSuccess/Error on coupon redemption.</v>
+      </c>
+      <c r="E122" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F122" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G122" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H122" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B123" t="str">
+        <v>01:30</v>
+      </c>
+      <c r="C123" t="str">
+        <v>src/services/storageService.ts</v>
+      </c>
+      <c r="D123" t="str">
+        <v>BL-034 (Sprint 4): exportBackupJSON() exports contacts+groups+drafts+settings as JSON with UTF-8 encoding; importBackupJSON() reads File and restores data after validation. Version and exportedAt metadata included.</v>
+      </c>
+      <c r="E123" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F123" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G123" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H123" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B124" t="str">
+        <v>01:30</v>
+      </c>
+      <c r="C124" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D124" t="str">
+        <v>BL-034 (Sprint 4): Added Backup and Restore buttons to Premium Features card. Hidden file input for restore. Success reloads page after 1.2s. Error feedback clears after 3s.</v>
+      </c>
+      <c r="E124" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F124" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G124" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H124" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B125" t="str">
+        <v>01:45</v>
+      </c>
+      <c r="C125" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D125" t="str">
+        <v>BL-035 (Sprint 4): Duplicate contact detection on new contact creation. findDuplicate() checks exact name match or phone (7+ digits stripped). Modal warns with matching name and offers "Save Anyway" or "Cancel". Edit mode excluded.</v>
+      </c>
+      <c r="E125" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F125" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G125" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H125" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B126" t="str">
+        <v>01:45</v>
+      </c>
+      <c r="C126" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D126" t="str">
+        <v>BL-024+034+035: Added 13 i18n keys in EN+HE: settings_backupData/Success, settings_restoreData/Success/Error, contactForm_duplicateTitle/Body/SaveAnyway.</v>
+      </c>
+      <c r="E126" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F126" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G126" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H126" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H120"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H126"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix changelog tracking: script now reads changelog_queue.json directly
Rewrote make-changelog.js to read from changelog_queue.json as the
single source of truth. 64 pre-queue legacy rows kept as LEGACY_ROWS
static array. All future entries only need changelog_queue.json — no
more editing the script.

Recovered 24 entries that existed in the queue but were never included
in changelog.xlsx. Total: 150 entries (was 125).

Going forward: agents append to changelog_queue.json → npm run changelog
regenerates xlsx automatically with zero manual edits to the script.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H126"/>
+  <dimension ref="A1:H151"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -1864,10 +1864,10 @@
         <v>10:00</v>
       </c>
       <c r="C66" t="str">
-        <v>src/integrations/supabase/client.ts, src/integrations/payment/payme.ts, src/integrations/ai/claudeClient.ts</v>
+        <v>src/integrations/supabase/client.ts</v>
       </c>
       <c r="D66" t="str">
-        <v>BUG-030: Add eslint-disable-next-line no-unused-vars to stub parameters (_userId, _req) in integration files to fix lint errors</v>
+        <v>תוקן BUG-030 — no-unused-vars lint על פרמטר _userId ב-stub; הוסף eslint-disable-next-line</v>
       </c>
       <c r="E66" t="str">
         <v>bugfix</v>
@@ -1887,13 +1887,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B67" t="str">
-        <v>10:30</v>
+        <v>10:00</v>
       </c>
       <c r="C67" t="str">
-        <v>src/screens/SettingsScreen.tsx</v>
+        <v>src/integrations/payment/payme.ts</v>
       </c>
       <c r="D67" t="str">
-        <v>BUG-031: Language toggle indicator invisible when Hebrew selected. Moved width/borderRadius from Tailwind arbitrary-value class (w-[calc(50%-4px)]) to inline style — Tailwind stripped the spaces in calc() generating invalid CSS</v>
+        <v>תוקן BUG-030 — no-unused-vars lint על פרמטר _req ב-stub; הוסף eslint-disable-next-line</v>
       </c>
       <c r="E67" t="str">
         <v>bugfix</v>
@@ -1902,7 +1902,7 @@
         <v>code_change</v>
       </c>
       <c r="G67" t="str">
-        <v>Agent 1</v>
+        <v>Agent 5</v>
       </c>
       <c r="H67" t="str">
         <v>done</v>
@@ -1913,22 +1913,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B68" t="str">
-        <v>11:00</v>
+        <v>10:00</v>
       </c>
       <c r="C68" t="str">
-        <v>src/components/WhatsAppButton.tsx</v>
+        <v>src/integrations/ai/claudeClient.ts</v>
       </c>
       <c r="D68" t="str">
-        <v>Add automatic image copy to clipboard on WhatsApp button click; Hebrew popup with paste instructions; close button; stores image as base64 canvas snapshot</v>
+        <v>תוקן BUG-030 — no-unused-vars lint על פרמטר _req ב-stub; הוסף eslint-disable-next-line</v>
       </c>
       <c r="E68" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F68" t="str">
         <v>code_change</v>
       </c>
       <c r="G68" t="str">
-        <v>Agent 1</v>
+        <v>Agent 5</v>
       </c>
       <c r="H68" t="str">
         <v>done</v>
@@ -1939,13 +1939,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B69" t="str">
-        <v>11:00</v>
+        <v>10:30</v>
       </c>
       <c r="C69" t="str">
-        <v>src/services/communicationService.ts</v>
+        <v>src/screens/SettingsScreen.tsx</v>
       </c>
       <c r="D69" t="str">
-        <v>BUG-032/033/034: Fix double 00-prefix in WhatsApp URL builder; add guard for empty phone string; remove deprecated execCommand clipboard fallback</v>
+        <v>תוקן BUG-031 — מחוון שפה בלתי נראה; w-[calc(50%-4px)] ב-Tailwind יצר CSS לא תקין; הועבר ל-inline style</v>
       </c>
       <c r="E69" t="str">
         <v>bugfix</v>
@@ -1965,13 +1965,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B70" t="str">
-        <v>11:30</v>
+        <v>11:00</v>
       </c>
       <c r="C70" t="str">
-        <v>src/screens/CalendarScreen.tsx</v>
+        <v>src/components/WhatsAppButton.tsx</v>
       </c>
       <c r="D70" t="str">
-        <v>Add @hebcal/core Hebrew date (gematria) to every calendar cell; Rosh Chodesh shows month name; Hebrew month names in pill badge</v>
+        <v>נוסף: העתקת תמונה אוטומטית ל-clipboard בלחיצה על WhatsApp; popup עברי עם הנחיות הדבקה; כפתור סיום</v>
       </c>
       <c r="E70" t="str">
         <v>feature</v>
@@ -1991,22 +1991,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B71" t="str">
-        <v>11:30</v>
+        <v>11:00</v>
       </c>
       <c r="C71" t="str">
-        <v>src/i18n/index.ts</v>
+        <v>src/services/communicationService.ts</v>
       </c>
       <c r="D71" t="str">
-        <v>Add 3 i18n keys: whatsapp_image_ready_title, whatsapp_image_paste_hint, whatsapp_image_paste_steps (EN + HE)</v>
+        <v>תוקן BUG-032 (00-prefix כפול), BUG-033 (guard טלפון ריק), BUG-034 (הוסר execCommand מיושן)</v>
       </c>
       <c r="E71" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F71" t="str">
         <v>code_change</v>
       </c>
       <c r="G71" t="str">
-        <v>Foundation-Agent</v>
+        <v>Agent 1</v>
       </c>
       <c r="H71" t="str">
         <v>done</v>
@@ -2017,16 +2017,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B72" t="str">
-        <v>12:00</v>
+        <v>11:30</v>
       </c>
       <c r="C72" t="str">
-        <v>AGENTS.md</v>
+        <v>src/screens/CalendarScreen.tsx</v>
       </c>
       <c r="D72" t="str">
-        <v>Create AGENTS.md — documentation of all 8 agent definitions, roles, and iteration action logs</v>
+        <v>נוסף: שילוב @hebcal/core — תאריך עברי (גמטריה) בכל תא; ראש חודש עם שם חודש; שמות חודשים עבריים ב-pill</v>
       </c>
       <c r="E72" t="str">
-        <v>improvement</v>
+        <v>feature</v>
       </c>
       <c r="F72" t="str">
         <v>code_change</v>
@@ -2043,13 +2043,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B73" t="str">
-        <v>15:00</v>
+        <v>11:30</v>
       </c>
       <c r="C73" t="str">
         <v>src/i18n/index.ts</v>
       </c>
       <c r="D73" t="str">
-        <v>Add 20 i18n keys: urgency_critical/high/medium/low, go_back, action_wish_birthday_today/days, action_wish_holiday_days, action_reconnect_days, action_checkin, action_followup, holiday_major, holiday_moreContacts (EN + HE)</v>
+        <v>נוספו 3 מפתחות i18n: whatsapp_image_ready_title, whatsapp_image_paste_hint, whatsapp_image_paste_steps (EN + HE)</v>
       </c>
       <c r="E73" t="str">
         <v>feature</v>
@@ -2069,16 +2069,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B74" t="str">
-        <v>15:00</v>
+        <v>12:00</v>
       </c>
       <c r="C74" t="str">
-        <v>src/core/scoringSystem.ts</v>
+        <v>AGENTS.md</v>
       </c>
       <c r="D74" t="str">
-        <v>BUG-020: Fix getBirthdayDaysUntil using date-fns differenceInCalendarDays — prevents wrong result on DST change days</v>
+        <v>נוצר AGENTS.md — תיעוד כל 8 agent הגדרות ופעולות מהפרויקט</v>
       </c>
       <c r="E74" t="str">
-        <v>bugfix</v>
+        <v>feature</v>
       </c>
       <c r="F74" t="str">
         <v>code_change</v>
@@ -2095,22 +2095,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B75" t="str">
-        <v>15:00</v>
+        <v>13:00</v>
       </c>
       <c r="C75" t="str">
-        <v>src/components/Navigation.tsx, src/screens/ContactDetailScreen.tsx, src/screens/HolidayDetailScreen.tsx, src/screens/DashboardScreen.tsx, src/screens/GroupsScreen.tsx, src/components/ui/Modal.tsx, src/screens/premium/ImportContactsScreen.tsx, src/components/ContactCard.tsx, src/index.css</v>
+        <v>BUG_REPORT.md</v>
       </c>
       <c r="D75" t="str">
-        <v>BUG-036 / FINDINGS 25A/20/23/28A/30B/60/66/67/69: aria-labels localized, urgency/frequency labels translated, group+dashboard cards converted to &lt;button&gt;, .btn:focus-visible ring added, setImporting in finally, decorative icon aria-hidden</v>
+        <v>עודכן בזמן אמת — BUG-022 סומן כ-fixed; נוספו BUG-030 עד BUG-035 עם תיאור מלא</v>
       </c>
       <c r="E75" t="str">
-        <v>bugfix</v>
+        <v>improvement</v>
       </c>
       <c r="F75" t="str">
         <v>code_change</v>
       </c>
       <c r="G75" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H75" t="str">
         <v>done</v>
@@ -2121,22 +2121,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B76" t="str">
-        <v>15:00</v>
+        <v>13:00</v>
       </c>
       <c r="C76" t="str">
-        <v>src/screens/SettingsScreen.tsx, src/screens/UpgradeScreen.tsx</v>
+        <v>agent_state/iteration_log.md</v>
       </c>
       <c r="D76" t="str">
-        <v>SECURITY: Wrap Danger Zone section and demo premium activation button in import.meta.env.DEV — both are completely tree-shaken from production builds by rolldown</v>
+        <v>נוסף iteration 11 — SettingsScreen/WhatsApp/communicationService/CalendarScreen/i18n/AGENTS.md</v>
       </c>
       <c r="E76" t="str">
-        <v>bugfix</v>
+        <v>improvement</v>
       </c>
       <c r="F76" t="str">
         <v>code_change</v>
       </c>
       <c r="G76" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H76" t="str">
         <v>done</v>
@@ -2147,13 +2147,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B77" t="str">
-        <v>16:00</v>
+        <v>13:30</v>
       </c>
       <c r="C77" t="str">
-        <v>src/utils/hebrewDateUtils.ts</v>
+        <v>agent_state/qa_status.json</v>
       </c>
       <c r="D77" t="str">
-        <v>Create hebrewDateUtils.ts — getHebrewDateStr(isoDate) converts Gregorian ISO date to Hebrew gematria string (e.g. ד׳ באייר תשפ״ו); uses local-time Date construction to avoid UTC timezone shifts</v>
+        <v>נוצר קובץ סטטוס QA עם 57 בדיקות — מצב נוכחי: 39 ✅ / 13 ❌ / 5 ⚠️</v>
       </c>
       <c r="E77" t="str">
         <v>feature</v>
@@ -2162,7 +2162,7 @@
         <v>code_change</v>
       </c>
       <c r="G77" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H77" t="str">
         <v>done</v>
@@ -2173,22 +2173,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B78" t="str">
-        <v>16:00</v>
+        <v>13:30</v>
       </c>
       <c r="C78" t="str">
-        <v>src/data/holidays.ts</v>
+        <v>scripts/make-qa-checklist.js</v>
       </c>
       <c r="D78" t="str">
-        <v>BUG-037: Yom HaAtzmaut 2026 was hardcoded as 2026-04-29 (wrong by 8 days); replaced with runtime computation via HebrewCalendar.getHolidaysForYearArray(5786, true) from @hebcal/core; correct date is 2026-04-21 (ד׳ באייר תשפ״ו)</v>
+        <v>נוצר סקריפט ליצירת NeverMiss_QA_Checklist.xlsx — קורא מ-qa_status.json; 57 בדיקות ב-8 קטגוריות</v>
       </c>
       <c r="E78" t="str">
-        <v>bugfix</v>
+        <v>feature</v>
       </c>
       <c r="F78" t="str">
         <v>code_change</v>
       </c>
       <c r="G78" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H78" t="str">
         <v>done</v>
@@ -2199,22 +2199,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B79" t="str">
-        <v>16:00</v>
+        <v>13:30</v>
       </c>
       <c r="C79" t="str">
-        <v>src/components/HolidayCard.tsx, src/screens/HolidayDetailScreen.tsx</v>
+        <v>package.json</v>
       </c>
       <c r="D79" t="str">
-        <v>Add Hebrew date badge (gematria format) to HolidayCard compact/full views and HolidayDetailScreen hero banner for all dateType === "hebrew" holidays</v>
+        <v>נוספו scripts: "changelog" → node scripts/make-changelog.js; "qa" → node scripts/make-qa-checklist.js</v>
       </c>
       <c r="E79" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F79" t="str">
         <v>code_change</v>
       </c>
       <c r="G79" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H79" t="str">
         <v>done</v>
@@ -2225,22 +2225,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B80" t="str">
-        <v>17:00</v>
+        <v>13:30</v>
       </c>
       <c r="C80" t="str">
-        <v>src/screens/TermsScreen.tsx</v>
+        <v>CLAUDE.md</v>
       </c>
       <c r="D80" t="str">
-        <v>BUG-038: Terms of Service page always showed English. Root cause: SECTIONS array was at module scope — t() calls were made once on load, ignoring language changes. Fix: moved SECTIONS inside component; replaced all hardcoded strings with titleKey/bodyKey references + t() calls with as const + TranslationKey cast</v>
+        <v>עודכן Quality Gate — נוספו שלבים 6-9: append changelog_queue, עדכון qa_status.json, הרצת changelog ו-qa</v>
       </c>
       <c r="E80" t="str">
-        <v>bugfix</v>
+        <v>improvement</v>
       </c>
       <c r="F80" t="str">
         <v>code_change</v>
       </c>
       <c r="G80" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H80" t="str">
         <v>done</v>
@@ -2251,13 +2251,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B81" t="str">
-        <v>17:00</v>
+        <v>13:30</v>
       </c>
       <c r="C81" t="str">
-        <v>src/i18n/index.ts</v>
+        <v>NeverMiss_QA_Checklist.xlsx</v>
       </c>
       <c r="D81" t="str">
-        <v>Add 22 i18n keys for Terms of Service: terms_lastUpdated, terms_intro, terms_s1_title/body through terms_s10_title/body — full Hebrew translations for all 10 sections (EN + HE)</v>
+        <v>נוצר NeverMiss_QA_Checklist.xlsx — 57 בדיקות ב-8 קטגוריות; מעודכן אוטומטית אחרי כל phase</v>
       </c>
       <c r="E81" t="str">
         <v>feature</v>
@@ -2266,7 +2266,7 @@
         <v>code_change</v>
       </c>
       <c r="G81" t="str">
-        <v>Foundation-Agent</v>
+        <v>Agent 4</v>
       </c>
       <c r="H81" t="str">
         <v>done</v>
@@ -2277,22 +2277,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B82" t="str">
-        <v>18:00</v>
+        <v>15:00</v>
       </c>
       <c r="C82" t="str">
-        <v>src/services/analyticsService.ts</v>
+        <v>src/i18n/index.ts</v>
       </c>
       <c r="D82" t="str">
-        <v>Create local analytics service: getAnonymousUserId() generates/persists UUID in localStorage (nm_user_id); trackEvent(name, metadata?) stores up to 100 events FIFO in nm_events. No backend, no dashboard, zero side effects.</v>
+        <v>נוספו 20 מפתחות i18n: urgency_critical/high/medium/low, go_back, action_wish_birthday_today/days, action_wish_holiday_days, action_reconnect_days, action_checkin, action_followup, holiday_major, holiday_moreContacts — EN + HE</v>
       </c>
       <c r="E82" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F82" t="str">
         <v>code_change</v>
       </c>
       <c r="G82" t="str">
-        <v>Agent 1</v>
+        <v>Foundation-Agent</v>
       </c>
       <c r="H82" t="str">
         <v>done</v>
@@ -2303,16 +2303,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B83" t="str">
-        <v>18:00</v>
+        <v>15:00</v>
       </c>
       <c r="C83" t="str">
-        <v>src/App.tsx, src/screens/ContactFormScreen.tsx, src/components/ChannelPicker.tsx, src/screens/premium/ImportContactsScreen.tsx</v>
+        <v>src/core/scoringSystem.ts</v>
       </c>
       <c r="D83" t="str">
-        <v>Add trackEvent calls for 4 events: app_open (AppShell mount), contact_created (new contact only), greeting_sent (with channel metadata), contacts_imported (with count metadata)</v>
+        <v>תוקן BUG-020 — getBirthdayDaysUntil עבר ל-differenceInCalendarDays מ-date-fns; מונע תוצאה שגויה בימי שינוי שעון</v>
       </c>
       <c r="E83" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F83" t="str">
         <v>code_change</v>
@@ -2329,13 +2329,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B84" t="str">
-        <v>19:00</v>
+        <v>15:00</v>
       </c>
       <c r="C84" t="str">
-        <v>src/screens/CalendarScreen.tsx</v>
+        <v>src/components/Navigation.tsx</v>
       </c>
       <c r="D84" t="str">
-        <v>BUG-039: Contact birthdays never appeared in calendar. Added birthdayMap useMemo — builds Map&lt;date-string, Contact[]&gt; for visible month using hebrewBirthday (priority) or birthday. Pink dot (#EC4899) added to cell dots row. Birthday panel section added below calendar showing contact name cards for selected day / full month.</v>
+        <v>תוקן FINDING 25A — PageHeader מוסיף useT(); aria-label="Go back" הוחלף ב-t('go_back') — עברית/אנגלית לפי שפה</v>
       </c>
       <c r="E84" t="str">
         <v>bugfix</v>
@@ -2355,16 +2355,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B85" t="str">
-        <v>19:00</v>
+        <v>15:00</v>
       </c>
       <c r="C85" t="str">
-        <v>src/types/index.ts</v>
+        <v>src/screens/ContactDetailScreen.tsx</v>
       </c>
       <c r="D85" t="str">
-        <v>FEATURE: Add optional hebrewBirthday?: string field to Contact interface — stored as "DD-MM" (Hebrew day-month, year-agnostic). Additive only; does not affect existing birthday field.</v>
+        <v>תוקן FINDING 20/23 — urgencyLevel מוצג עם t(); interactionFrequency עם t(); translatedActionLabel IIFE לפי action.type</v>
       </c>
       <c r="E85" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F85" t="str">
         <v>code_change</v>
@@ -2381,16 +2381,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B86" t="str">
-        <v>19:00</v>
+        <v>15:00</v>
       </c>
       <c r="C86" t="str">
-        <v>src/utils/hebrewDateUtils.ts</v>
+        <v>src/screens/HolidayDetailScreen.tsx</v>
       </c>
       <c r="D86" t="str">
-        <v>FEATURE: Add hebrewBirthdayToGregorianInCalendarYear(hebrewBirthday, gregorianYear) — converts "DD-MM" Hebrew date to Gregorian Date for a given year; tries approxHYear and approxHYear+1 to handle year boundary; returns null for invalid combos (e.g. Adar II in non-leap year)</v>
+        <v>תוקן FINDING 28A — ★ Major הוחלף ב-t('holiday_major'); +N more contacts הוחלף ב-t('holiday_moreContacts', { n })</v>
       </c>
       <c r="E86" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F86" t="str">
         <v>code_change</v>
@@ -2407,16 +2407,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B87" t="str">
-        <v>19:00</v>
+        <v>15:00</v>
       </c>
       <c r="C87" t="str">
-        <v>src/screens/ContactFormScreen.tsx</v>
+        <v>src/screens/DashboardScreen.tsx</v>
       </c>
       <c r="D87" t="str">
-        <v>FEATURE: Add Hebrew Birthday UI in premium section — shown for Judaism contacts or when hebrewBirthday already set. Two dropdowns (day 1–30, Hebrew month 1–12 with names). Derives day/month from form.hebrewBirthday via useMemo. Clear button removes the field. Saved as "DD-MM" string.</v>
+        <v>תוקן FINDING 67 — Today highlight cards (holiday + birthday) הומרו מ-div ל-&lt;button type=button&gt; עם w-full text-left</v>
       </c>
       <c r="E87" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F87" t="str">
         <v>code_change</v>
@@ -2433,22 +2433,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B88" t="str">
-        <v>19:00</v>
+        <v>15:00</v>
       </c>
       <c r="C88" t="str">
-        <v>src/i18n/index.ts</v>
+        <v>src/screens/GroupsScreen.tsx</v>
       </c>
       <c r="D88" t="str">
-        <v>Add 7 i18n keys (EN + HE): calendar_birthdays, calendar_birthdayLabel, calendar_birthdaysOn, contactForm_hebrewBirthday, contactForm_hebrewBirthdayDay, contactForm_hebrewBirthdayMonth, contactForm_hebrewBirthdayClear</v>
+        <v>תוקן FINDING 67 — Group card הומר מ-div ל-&lt;button type=button&gt; עם w-full text-left</v>
       </c>
       <c r="E88" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F88" t="str">
         <v>code_change</v>
       </c>
       <c r="G88" t="str">
-        <v>Foundation-Agent</v>
+        <v>Agent 1</v>
       </c>
       <c r="H88" t="str">
         <v>done</v>
@@ -2459,16 +2459,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B89" t="str">
-        <v>20:00</v>
+        <v>15:00</v>
       </c>
       <c r="C89" t="str">
-        <v>src/screens/GreetingEditorScreen.tsx</v>
+        <v>src/index.css</v>
       </c>
       <c r="D89" t="str">
-        <v>BL-015: Replace hardcoded tier desc strings with i18n keys (greeting_tier_*_desc). Signature placeholder via t('greeting_signature_placeholder'). BL-017: aria-label on Regenerate and Copy icon buttons. BL-018: aria-expanded on Advanced tone + Signature toggle buttons. aria-hidden on decorative icons.</v>
+        <v>תוקן FINDING 69 — נוסף .btn:focus-visible { outline: 2px solid var(--color-primary) }; נוסף @media (min-width: 768px) שמסיר max-width:480px על דסקטופ</v>
       </c>
       <c r="E89" t="str">
-        <v>improvement</v>
+        <v>bugfix</v>
       </c>
       <c r="F89" t="str">
         <v>code_change</v>
@@ -2485,22 +2485,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B90" t="str">
-        <v>20:00</v>
+        <v>15:00</v>
       </c>
       <c r="C90" t="str">
-        <v>src/i18n/index.ts</v>
+        <v>src/components/ui/Modal.tsx</v>
       </c>
       <c r="D90" t="str">
-        <v>BL-015: Add 4 i18n keys (EN + HE): greeting_tier_casual_desc, greeting_tier_professional_desc, greeting_tier_vip_desc, greeting_signature_placeholder</v>
+        <v>תוקן FINDING 30B — Modal מייבא useT(); aria-label='Close' הוחלף ב-t('close') — עברית/אנגלית לפי שפה</v>
       </c>
       <c r="E90" t="str">
-        <v>improvement</v>
+        <v>bugfix</v>
       </c>
       <c r="F90" t="str">
         <v>code_change</v>
       </c>
       <c r="G90" t="str">
-        <v>Foundation-Agent</v>
+        <v>Agent 1</v>
       </c>
       <c r="H90" t="str">
         <v>done</v>
@@ -2511,16 +2511,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B91" t="str">
-        <v>20:00</v>
+        <v>15:00</v>
       </c>
       <c r="C91" t="str">
-        <v>src/components/ContactCard.tsx</v>
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
       </c>
       <c r="D91" t="str">
-        <v>BL-016: Add ACTION_KEY Record&lt;SuggestedActionType, TranslationKey&gt; map. Use useT() + t(ACTION_KEY[...]) to display action label in current language instead of raw English label string.</v>
+        <v>תוקן FINDING 60 — setImporting(false) הועבר ל-finally block; מניעת Import button תקוע במצב loading</v>
       </c>
       <c r="E91" t="str">
-        <v>improvement</v>
+        <v>bugfix</v>
       </c>
       <c r="F91" t="str">
         <v>code_change</v>
@@ -2537,16 +2537,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B92" t="str">
-        <v>20:00</v>
+        <v>15:00</v>
       </c>
       <c r="C92" t="str">
-        <v>src/screens/ContactDetailScreen.tsx</v>
+        <v>src/components/ContactCard.tsx</v>
       </c>
       <c r="D92" t="str">
-        <v>BL-017: aria-label on Edit icon button via t('contactForm_edit'). BL-041: Add celebration feedback on Mark as Contacted — 6 emoji particle burst (.animate-particle with --tx/--ty CSS vars), Web Audio oscillator ping (880→1200Hz ramp, 0.4s), haptic navigator.vibrate(40). Respects prefers-reduced-motion. useState celebrating moved before early return to comply with hooks rules.</v>
+        <v>תוקן FINDING 66 — aria-hidden="true" נוסף ל-Crown ו-Building2 icons; אלמנטים דקורטיביים מוסתרים מקורא מסך</v>
       </c>
       <c r="E92" t="str">
-        <v>improvement</v>
+        <v>bugfix</v>
       </c>
       <c r="F92" t="str">
         <v>code_change</v>
@@ -2563,13 +2563,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B93" t="str">
-        <v>20:00</v>
+        <v>15:00</v>
       </c>
       <c r="C93" t="str">
-        <v>src/index.css</v>
+        <v>agent_state/qa_status.json</v>
       </c>
       <c r="D93" t="str">
-        <v>BL-041: Add @keyframes particleBurst (translate + scale to 0 + opacity fade driven by --tx/--ty CSS custom properties) and .animate-particle utility class (1.2s ease-out forwards).</v>
+        <v>עודכן — T05/T07/T08/T09/T10/T39/T40/T41/T42/T45/T46/T48 סומנו כ-✅; 8 בדיקות תוקנו ב-iteration 12</v>
       </c>
       <c r="E93" t="str">
         <v>improvement</v>
@@ -2578,7 +2578,7 @@
         <v>code_change</v>
       </c>
       <c r="G93" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H93" t="str">
         <v>done</v>
@@ -2589,22 +2589,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B94" t="str">
-        <v>20:30</v>
+        <v>16:00</v>
       </c>
       <c r="C94" t="str">
-        <v>agent_state/iteration_log.md</v>
+        <v>src/utils/hebrewDateUtils.ts</v>
       </c>
       <c r="D94" t="str">
-        <v>BUG-040 fix: reconstructed iterations 13–17 from changelog_queue.json. All 5 entries appended: iter 13 (Hebrew date display + BUG-037), iter 14 (BUG-038 Terms fix), iter 15 (analytics foundation), iter 16 (BUG-039 birthday calendar + Hebrew birthday feature), iter 17 (BL-015/016/017/018/041 i18n + accessibility + celebration). Agent 2/3 columns marked TBD where source files have no entries. Log is now continuous 0–17.</v>
+        <v>נוצר util חדש — getHebrewDateStr() מחזיר תאריך עברי בגימטריה: ד׳ באייר תשפ״ו; משתמש ב-HDate + gematriya מ-@hebcal/core</v>
       </c>
       <c r="E94" t="str">
-        <v>bugfix</v>
+        <v>feature</v>
       </c>
       <c r="F94" t="str">
         <v>code_change</v>
       </c>
       <c r="G94" t="str">
-        <v>Agent 4</v>
+        <v>Agent 1</v>
       </c>
       <c r="H94" t="str">
         <v>done</v>
@@ -2615,13 +2615,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B95" t="str">
-        <v>20:30</v>
+        <v>16:00</v>
       </c>
       <c r="C95" t="str">
-        <v>BUG_REPORT.md</v>
+        <v>src/data/holidays.ts</v>
       </c>
       <c r="D95" t="str">
-        <v>Added BUG-040 entry: iteration_log.md missing iterations 13–17. Marked fixed.</v>
+        <v>תוקן BUG-037 — יום העצמאות 2026 היה מקודד כ-2026-04-29 (שגוי); כעת מחושב בזמן ריצה ע"י HebrewCalendar.getHolidaysForYearArray(5786) מ-@hebcal/core; התוצאה: 2026-04-21 (ד׳ באייר תשפ"ו)</v>
       </c>
       <c r="E95" t="str">
         <v>bugfix</v>
@@ -2630,7 +2630,7 @@
         <v>code_change</v>
       </c>
       <c r="G95" t="str">
-        <v>Agent 4</v>
+        <v>Agent 1</v>
       </c>
       <c r="H95" t="str">
         <v>done</v>
@@ -2641,13 +2641,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B96" t="str">
-        <v>21:00</v>
+        <v>16:00</v>
       </c>
       <c r="C96" t="str">
-        <v>src/App.tsx</v>
+        <v>src/components/HolidayCard.tsx</v>
       </c>
       <c r="D96" t="str">
-        <v>BL-019: Convert 13 screens to React.lazy (CalendarScreen, HolidayDetailScreen, ContactsScreen, ContactDetailScreen, ContactFormScreen, GreetingEditorScreen, GroupsScreen, SettingsScreen, UpgradeScreen, AboutScreen, PrivacyScreen, TermsScreen, WhatsNewScreen). Move Suspense fallback into WithNav so BottomNav stays visible during load. Remove now-redundant inner Suspense from 3 premium routes. Main bundle: 435 kB → 285 kB raw (-150 kB), 130 kB → 93 kB gzip (-37 kB).</v>
+        <v>נוסף תצוגת תאריך עברי לחגים יהודיים (dateType === 'hebrew') — כרטיס קומפקטי ומלא; פורמט: ד׳ באייר תשפ״ו</v>
       </c>
       <c r="E96" t="str">
         <v>improvement</v>
@@ -2667,13 +2667,25 @@
         <v>2026-04-28</v>
       </c>
       <c r="B97" t="str">
-        <v>21:00</v>
+        <v>16:00</v>
       </c>
       <c r="C97" t="str">
-        <v>src/core/scoringSystem.ts</v>
+        <v>src/screens/HolidayDetailScreen.tsx</v>
       </c>
       <c r="D97" t="str">
-        <v>BL-020: Add module-level scoreCache Map&lt;string, RelationshipScore&gt; keyed by `contact.id|contact.updatedAt`. calculateRelationshipScore checks cache on entry and sets result before return. Eliminates redundant scoring for unchanged contacts on every render. Stale results impossible since updatedAt is always stamped on mutation.</v>
+        <v>נוסף badge תאריך עברי בבאנר הראשי של מסך פרטי החג; מוצג רק לחגים עם dateType === 'hebrew'</v>
+      </c>
+      <c r="E97" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F97" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H97" t="str">
+        <v>done</v>
       </c>
     </row>
     <row r="98">
@@ -2681,22 +2693,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B98" t="str">
-        <v>22:00</v>
+        <v>17:00</v>
       </c>
       <c r="C98" t="str">
-        <v>src/types/index.ts</v>
+        <v>src/screens/TermsScreen.tsx</v>
       </c>
       <c r="D98" t="str">
-        <v>BL-026: Add CelebrationType union type (Jewish|Christian|Muslim|Druze|Secular); add optional celebrationType field to Contact interface</v>
+        <v>תוקן BUG-038 — מסך תנאי שירות הציג תמיד אנגלית; SECTIONS הועבר לתוך הקומפוננטה עם t(); כל 10 כותרות + גופי סעיפים + כותרת הגיבור + תאריך עדכון + טקסט מבוא כעת דינמיים</v>
       </c>
       <c r="E98" t="str">
-        <v>feature</v>
+        <v>bugfix</v>
       </c>
       <c r="F98" t="str">
         <v>code_change</v>
       </c>
       <c r="G98" t="str">
-        <v>Foundation Agent</v>
+        <v>Agent 1</v>
       </c>
       <c r="H98" t="str">
         <v>done</v>
@@ -2707,22 +2719,22 @@
         <v>2026-04-28</v>
       </c>
       <c r="B99" t="str">
-        <v>22:00</v>
+        <v>17:00</v>
       </c>
       <c r="C99" t="str">
         <v>src/i18n/index.ts</v>
       </c>
       <c r="D99" t="str">
-        <v>BL-026+BL-023+BL-030: Add 34 i18n keys — celebrationType_* (5 values EN+HE), contactForm_celebrationType, notif_overdue/notif_overdue_body, 14 deviceContacts_* keys, premium_feat_device_contacts — all in EN and HE</v>
+        <v>נוספו 22 מפתחות i18n לתנאי שירות: terms_lastUpdated, terms_intro, terms_s1_title/body עד terms_s10_title/body — בעברית ובאנגלית</v>
       </c>
       <c r="E99" t="str">
-        <v>improvement</v>
+        <v>feature</v>
       </c>
       <c r="F99" t="str">
         <v>code_change</v>
       </c>
       <c r="G99" t="str">
-        <v>Foundation Agent</v>
+        <v>Foundation-Agent</v>
       </c>
       <c r="H99" t="str">
         <v>done</v>
@@ -2733,13 +2745,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B100" t="str">
-        <v>22:00</v>
+        <v>18:00</v>
       </c>
       <c r="C100" t="str">
-        <v>src/core/scoringSystem.ts</v>
+        <v>src/services/analyticsService.ts</v>
       </c>
       <c r="D100" t="str">
-        <v>BL-026: Add CELEBRATION_TO_RELIGION map; update getUpcomingHolidaysForContact to prefer celebrationType over religion when set, falling back to religion for existing contacts</v>
+        <v>נוסף שירות analytics מקומי: getAnonymousUserId() (localStorage nm_user_id), trackEvent(name, metadata?) — שומר עד 100 אירועים ב-FIFO ב-nm_events; ללא backend</v>
       </c>
       <c r="E100" t="str">
         <v>feature</v>
@@ -2759,16 +2771,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B101" t="str">
-        <v>22:00</v>
+        <v>18:00</v>
       </c>
       <c r="C101" t="str">
-        <v>src/screens/ContactFormScreen.tsx</v>
+        <v>src/App.tsx</v>
       </c>
       <c r="D101" t="str">
-        <v>BL-026: Add celebrationType Select dropdown to Cultural &amp; Language section; wire into form state and handleSave; import CelebrationType type</v>
+        <v>נוסף מעקב app_open ב-AppShell useEffect — מופעל פעם אחת בטעינת האפליקציה</v>
       </c>
       <c r="E101" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F101" t="str">
         <v>code_change</v>
@@ -2785,16 +2797,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B102" t="str">
-        <v>22:00</v>
+        <v>18:00</v>
       </c>
       <c r="C102" t="str">
-        <v>src/services/notificationService.ts</v>
+        <v>src/screens/ContactFormScreen.tsx</v>
       </c>
       <c r="D102" t="str">
-        <v>BL-023: Add overdue-contact reminder — fires when daysSince &gt;= 45 days with no upcoming birthday within 7 days; dedup via existing nm_notif_sent localStorage mechanism</v>
+        <v>נוסף מעקב contact_created לאחר addContact() ביצירת איש קשר חדש בלבד (לא בעדכון)</v>
       </c>
       <c r="E102" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F102" t="str">
         <v>code_change</v>
@@ -2811,16 +2823,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B103" t="str">
-        <v>22:00</v>
+        <v>18:00</v>
       </c>
       <c r="C103" t="str">
-        <v>src/screens/DeviceContactsScreen.tsx</v>
+        <v>src/components/ChannelPicker.tsx</v>
       </c>
       <c r="D103" t="str">
-        <v>BL-030: New screen — consent → permission request → device contact list with checkboxes → import with phone dedup. Capacitor.isNativePlatform() guard shows graceful web-only message. Imports @capacitor-community/contacts. Premium-gated via App.tsx route.</v>
+        <v>נוסף מעקב greeting_sent עם metadata { channel } בכל שליחת ברכה דרך כל ערוץ</v>
       </c>
       <c r="E103" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F103" t="str">
         <v>code_change</v>
@@ -2837,16 +2849,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B104" t="str">
-        <v>22:00</v>
+        <v>18:00</v>
       </c>
       <c r="C104" t="str">
-        <v>src/App.tsx</v>
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
       </c>
       <c r="D104" t="str">
-        <v>BL-030: Add DeviceContactsScreen lazy import; add route /device-contacts with Premium gate (isPremium ? DeviceContactsScreen : UpgradeScreen)</v>
+        <v>נוסף מעקב contacts_imported עם metadata { count } לאחר ייבוא אנשי קשר מוצלח</v>
       </c>
       <c r="E104" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F104" t="str">
         <v>code_change</v>
@@ -2863,16 +2875,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B105" t="str">
-        <v>22:00</v>
+        <v>19:00</v>
       </c>
       <c r="C105" t="str">
-        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+        <v>src/screens/CalendarScreen.tsx</v>
       </c>
       <c r="D105" t="str">
-        <v>BL-030: Add "Import from Phone" shortcut card at top of Import screen; navigates to /device-contacts</v>
+        <v>תוקן BUG-039 — ימי הולדת לא הוצגו בלוח השנה; נוסף birthdayMap useMemo; נוספת נקודה ורודה (#EC4899) על תאים עם ימי הולדת; נוסף פאנל 'ימי הולדת' עם שמות אנשי קשר</v>
       </c>
       <c r="E105" t="str">
-        <v>improvement</v>
+        <v>bugfix</v>
       </c>
       <c r="F105" t="str">
         <v>code_change</v>
@@ -2889,16 +2901,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B106" t="str">
-        <v>23:00</v>
+        <v>19:00</v>
       </c>
       <c r="C106" t="str">
-        <v>src/screens/CalendarScreen.tsx</v>
+        <v>src/types/index.ts</v>
       </c>
       <c r="D106" t="str">
-        <v>BUG-043: Fix multi-day holidays only showing dot on first day. Replace isSameDay check with numeric YYYYMMDD range [startNum, endNum] in getHolidaysForDay. Fix monthly list to show holidays overlapping the visible month (not just holidays that start in the month). Remove unused isSameMonth import.</v>
+        <v>נוסף שדה hebrewBirthday?: string לממשק Contact — פורמט 'DD-MM' (יום-חודש עברי ללא שנה)</v>
       </c>
       <c r="E106" t="str">
-        <v>bugfix</v>
+        <v>improvement</v>
       </c>
       <c r="F106" t="str">
         <v>code_change</v>
@@ -2915,16 +2927,16 @@
         <v>2026-04-28</v>
       </c>
       <c r="B107" t="str">
-        <v>23:00</v>
+        <v>19:00</v>
       </c>
       <c r="C107" t="str">
-        <v>src/data/holidays.ts</v>
+        <v>src/utils/hebrewDateUtils.ts</v>
       </c>
       <c r="D107" t="str">
-        <v>BUG-044: Add missing sukkot-2026 entry (Sep 25 – Oct 2, 2026 / 15–22 Tishrei 5787). Covers full festival including Hoshana Rabbah and Shemini Atzeret / Simchat Torah. Matches existing sukkot-2025 pattern.</v>
+        <v>נוספה פונקציה hebrewBirthdayToGregorianInCalendarYear() — ממירה 'DD-MM' עברי לתאריך גרגוריאני בשנה נתונה; בודקת שתי שנות היברו סמוכות</v>
       </c>
       <c r="E107" t="str">
-        <v>bugfix</v>
+        <v>improvement</v>
       </c>
       <c r="F107" t="str">
         <v>code_change</v>
@@ -2941,13 +2953,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B108" t="str">
-        <v>23:30</v>
+        <v>19:00</v>
       </c>
       <c r="C108" t="str">
-        <v>src/screens/ContactDetailScreen.tsx</v>
+        <v>src/screens/ContactFormScreen.tsx</v>
       </c>
       <c r="D108" t="str">
-        <v>BL-045: Replace harsh oscillator with C5/E5/G5 major triad arpeggio (3 sine waves, ~0.75s, pleasant chord). Expand particles from 6 to 10, size text-xl (was text-base), wider spread ±85px h / ±110px v. Animation delay stagger 50ms per particle (was 40ms). State clear timeout 1600ms.</v>
+        <v>נוסף UI לתאריך לידה עברי בסעיף פרמיום — מוצג לאנשי קשר יהודים או כשהשדה כבר מוגדר; שני dropdowns (יום + חודש עברי) + כפתור ניקוי</v>
       </c>
       <c r="E108" t="str">
         <v>improvement</v>
@@ -2967,13 +2979,13 @@
         <v>2026-04-28</v>
       </c>
       <c r="B109" t="str">
-        <v>23:30</v>
+        <v>19:00</v>
       </c>
       <c r="C109" t="str">
-        <v>src/index.css</v>
+        <v>src/i18n/index.ts</v>
       </c>
       <c r="D109" t="str">
-        <v>BL-045: Update particleBurst keyframe — scale-pop effect: 0.4 → 1.6 → 0 across 0/18%/100% keyframe stops, giving a visible "pop then fly" motion. Animation class duration 1.2s → 1.4s.</v>
+        <v>נוספו 7 מפתחות i18n: calendar_birthdays, calendar_birthdayLabel, calendar_birthdaysOn, contactForm_hebrewBirthday, contactForm_hebrewBirthdayDay, contactForm_hebrewBirthdayMonth, contactForm_hebrewBirthdayClear — EN + HE</v>
       </c>
       <c r="E109" t="str">
         <v>improvement</v>
@@ -2982,7 +2994,7 @@
         <v>code_change</v>
       </c>
       <c r="G109" t="str">
-        <v>Agent 1</v>
+        <v>Foundation-Agent</v>
       </c>
       <c r="H109" t="str">
         <v>done</v>
@@ -2990,19 +3002,19 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B110" t="str">
-        <v>00:00</v>
+        <v>20:00</v>
       </c>
       <c r="C110" t="str">
-        <v>src/services/exportService.ts</v>
+        <v>src/screens/GreetingEditorScreen.tsx</v>
       </c>
       <c r="D110" t="str">
-        <v>BL-025 (Sprint 4): New exportContactsToCSV() using PapaParse. Exports all Contact fields to CSV with UTF-8 BOM for Hebrew Excel compatibility. Downloads as nevermiss-contacts-YYYY-MM-DD.csv.</v>
+        <v>BL-015: החלפת תיאורי tier קשיחים ב-i18n (greeting_tier_*_desc); placeholder חתימה דרך t('greeting_signature_placeholder'); aria-label על כפתורי Regenerate ו-Copy; aria-expanded על toggles</v>
       </c>
       <c r="E110" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F110" t="str">
         <v>code_change</v>
@@ -3016,19 +3028,19 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B111" t="str">
-        <v>00:00</v>
+        <v>20:00</v>
       </c>
       <c r="C111" t="str">
-        <v>src/screens/SettingsScreen.tsx</v>
+        <v>src/components/ContactCard.tsx</v>
       </c>
       <c r="D111" t="str">
-        <v>BL-025 (Sprint 4): Added Export Contacts to CSV button in Premium Features card. exportDone state shows success feedback for 2.5s.</v>
+        <v>BL-016: תרגום תיאור פעולה מוצעת — ACTION_KEY map מ-SuggestedActionType ל-TranslationKey; שימוש ב-t() במקום label גולמי</v>
       </c>
       <c r="E111" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F111" t="str">
         <v>code_change</v>
@@ -3042,19 +3054,19 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B112" t="str">
-        <v>00:00</v>
+        <v>20:00</v>
       </c>
       <c r="C112" t="str">
-        <v>src/i18n/index.ts</v>
+        <v>src/screens/ContactDetailScreen.tsx</v>
       </c>
       <c r="D112" t="str">
-        <v>BL-025 (Sprint 4): Added i18n keys settings_exportContacts + settings_exportSuccess in EN+HE.</v>
+        <v>BL-017/018: aria-label על כפתור עריכה; BL-041: אנימציית פרטיקלים (6 אמוג'ים), צליל Web Audio (880→1200Hz), haptic navigator.vibrate(40) בלחיצה על 'סימון כיצרנו קשר'; תומך prefers-reduced-motion</v>
       </c>
       <c r="E112" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F112" t="str">
         <v>code_change</v>
@@ -3068,16 +3080,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B113" t="str">
-        <v>00:30</v>
+        <v>20:00</v>
       </c>
       <c r="C113" t="str">
-        <v>src/components/Navigation.tsx</v>
+        <v>src/i18n/index.ts</v>
       </c>
       <c r="D113" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Back button in PageHeader changed to min-w/h-[48px] flex items-center justify-center — 48×48px minimum tap target.</v>
+        <v>BL-015: נוספו מפתחות greeting_tier_casual_desc, greeting_tier_professional_desc, greeting_tier_vip_desc, greeting_signature_placeholder — EN + HE</v>
       </c>
       <c r="E113" t="str">
         <v>improvement</v>
@@ -3086,7 +3098,7 @@
         <v>code_change</v>
       </c>
       <c r="G113" t="str">
-        <v>Agent 1</v>
+        <v>Foundation-Agent</v>
       </c>
       <c r="H113" t="str">
         <v>done</v>
@@ -3094,16 +3106,16 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B114" t="str">
-        <v>00:30</v>
+        <v>20:00</v>
       </c>
       <c r="C114" t="str">
-        <v>src/screens/ContactFormScreen.tsx</v>
+        <v>src/index.css</v>
       </c>
       <c r="D114" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Delete icon button in ContactForm PageHeader changed to min-w/h-[48px] tap target.</v>
+        <v>BL-041: נוספה keyframe particleBurst ו-class .animate-particle לאנימציית פרטיקלים בחגיגה</v>
       </c>
       <c r="E114" t="str">
         <v>improvement</v>
@@ -3120,25 +3132,25 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B115" t="str">
-        <v>00:30</v>
+        <v>20:30</v>
       </c>
       <c r="C115" t="str">
-        <v>src/screens/GroupsScreen.tsx</v>
+        <v>agent_state/iteration_log.md</v>
       </c>
       <c r="D115" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Edit and Delete icon buttons on group cards changed to min-w/h-[48px] tap targets.</v>
+        <v>תוקן BUG-040 — iteration_log.md חסר iterations 13–17; שוחזרו מ-changelog_queue.json; עמודות Agent 2/3 סומנו TBD היכן שאין רשומות; הלוג רציף 0–17</v>
       </c>
       <c r="E115" t="str">
-        <v>improvement</v>
+        <v>bugfix</v>
       </c>
       <c r="F115" t="str">
         <v>code_change</v>
       </c>
       <c r="G115" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H115" t="str">
         <v>done</v>
@@ -3146,16 +3158,16 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B116" t="str">
-        <v>00:30</v>
+        <v>20:30</v>
       </c>
       <c r="C116" t="str">
-        <v>src/screens/GreetingEditorScreen.tsx</v>
+        <v>BUG_REPORT.md</v>
       </c>
       <c r="D116" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Regenerate and Copy icon buttons changed to min-w/h-[48px] tap targets.</v>
+        <v>נוסף BUG-040 — iteration_log.md חסר iterations 13–17; סומן כ-fixed</v>
       </c>
       <c r="E116" t="str">
         <v>improvement</v>
@@ -3164,7 +3176,7 @@
         <v>code_change</v>
       </c>
       <c r="G116" t="str">
-        <v>Agent 1</v>
+        <v>Agent 4</v>
       </c>
       <c r="H116" t="str">
         <v>done</v>
@@ -3172,16 +3184,16 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B117" t="str">
-        <v>00:30</v>
+        <v>21:00</v>
       </c>
       <c r="C117" t="str">
-        <v>src/components/ui/Modal.tsx</v>
+        <v>src/App.tsx</v>
       </c>
       <c r="D117" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Close (X) button in Modal header changed to min-w/h-[48px] tap target.</v>
+        <v>BL-019: 13 מסכים הומרו ל-React.lazy; Suspense נוסף בתוך WithNav; inner Suspense הוסר מנתיבי premium; bundle ראשי ירד מ-435kB ל-285kB</v>
       </c>
       <c r="E117" t="str">
         <v>improvement</v>
@@ -3198,16 +3210,16 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B118" t="str">
-        <v>00:30</v>
+        <v>21:00</v>
       </c>
       <c r="C118" t="str">
-        <v>src/screens/ContactDetailScreen.tsx</v>
+        <v>src/core/scoringSystem.ts</v>
       </c>
       <c r="D118" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Edit icon button in ContactDetail PageHeader changed to min-w/h-[48px] tap target.</v>
+        <v>BL-020: נוסף Map cache (scoreCache) ברמת המודול; מפתח: id|updatedAt; תוצאה נשמרת ומוחזרת מהמטמון לאנשי קשר שלא השתנו</v>
       </c>
       <c r="E118" t="str">
         <v>improvement</v>
@@ -3224,16 +3236,16 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B119" t="str">
-        <v>00:30</v>
+        <v>22:00</v>
       </c>
       <c r="C119" t="str">
-        <v>src/screens/HolidayDetailScreen.tsx</v>
+        <v>src/types/index.ts</v>
       </c>
       <c r="D119" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Copy greeting icon button changed to min-w/h-[48px] tap target.</v>
+        <v>BL-026: נוסף סוג CelebrationType (Jewish/Christian/Muslim/Druze/Secular) + שדה celebrationType? על Contact interface</v>
       </c>
       <c r="E119" t="str">
         <v>improvement</v>
@@ -3242,7 +3254,7 @@
         <v>code_change</v>
       </c>
       <c r="G119" t="str">
-        <v>Agent 1</v>
+        <v>FoundationAgent</v>
       </c>
       <c r="H119" t="str">
         <v>done</v>
@@ -3250,16 +3262,16 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B120" t="str">
-        <v>00:30</v>
+        <v>22:00</v>
       </c>
       <c r="C120" t="str">
-        <v>src/screens/premium/BirthdayGreetingEditorScreen.tsx</v>
+        <v>src/i18n/index.ts</v>
       </c>
       <c r="D120" t="str">
-        <v>BL-029 (Sprint 4) WCAG 2.5.5: Regenerate and Copy icon buttons in BirthdayGreetingEditor changed to min-w/h-[48px] tap targets.</v>
+        <v>BL-026+BL-023+BL-030: נוספו 34 מפתחות i18n — celebrationType_*, contactForm_celebrationType, notif_overdue/body, deviceContacts_*, premium_feat_device_contacts — EN+HE</v>
       </c>
       <c r="E120" t="str">
         <v>improvement</v>
@@ -3268,7 +3280,7 @@
         <v>code_change</v>
       </c>
       <c r="G120" t="str">
-        <v>Agent 1</v>
+        <v>FoundationAgent</v>
       </c>
       <c r="H120" t="str">
         <v>done</v>
@@ -3276,19 +3288,19 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B121" t="str">
-        <v>01:00</v>
+        <v>22:00</v>
       </c>
       <c r="C121" t="str">
-        <v>src/services/hapticService.ts</v>
+        <v>src/core/scoringSystem.ts</v>
       </c>
       <c r="D121" t="str">
-        <v>BL-024 (Sprint 4): New hapticService with hapticLight/Medium/Success/Error. Uses Capacitor.isNativePlatform() guard — graceful no-op in browser. ImpactStyle.Light/Medium and NotificationType.Success/Error.</v>
+        <v>BL-026: נוסף CELEBRATION_TO_RELIGION map; getUpcomingHolidaysForContact עכשיו מסנן לפי celebrationType כאשר מוגדר, נופל בחזרה ל-religion</v>
       </c>
       <c r="E121" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F121" t="str">
         <v>code_change</v>
@@ -3302,19 +3314,19 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B122" t="str">
-        <v>01:00</v>
+        <v>22:00</v>
       </c>
       <c r="C122" t="str">
-        <v>src/screens/ContactFormScreen.tsx + src/components/ChannelPicker.tsx + src/screens/UpgradeScreen.tsx</v>
+        <v>src/screens/ContactFormScreen.tsx</v>
       </c>
       <c r="D122" t="str">
-        <v>BL-024 (Sprint 4): Haptic wired to 3 key actions — hapticSuccess after contact save, hapticMedium on greeting channel select, hapticSuccess/Error on coupon redemption.</v>
+        <v>BL-026: נוסף select לסוג חגיגה בקטע תרבות (Cultural); celebrationType עובר ל-handleSave</v>
       </c>
       <c r="E122" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F122" t="str">
         <v>code_change</v>
@@ -3328,19 +3340,19 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B123" t="str">
-        <v>01:30</v>
+        <v>22:00</v>
       </c>
       <c r="C123" t="str">
-        <v>src/services/storageService.ts</v>
+        <v>src/services/notificationService.ts</v>
       </c>
       <c r="D123" t="str">
-        <v>BL-034 (Sprint 4): exportBackupJSON() exports contacts+groups+drafts+settings as JSON with UTF-8 encoding; importBackupJSON() reads File and restores data after validation. Version and exportedAt metadata included.</v>
+        <v>BL-023: נוספה התראת overdue — נשלחת כאשר daysSince &gt;= 45 ואין יום הולדת בקרוב (בעוד 7 ימים); dedup קיים דרך nm_notif_sent</v>
       </c>
       <c r="E123" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F123" t="str">
         <v>code_change</v>
@@ -3354,16 +3366,16 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B124" t="str">
-        <v>01:30</v>
+        <v>22:00</v>
       </c>
       <c r="C124" t="str">
-        <v>src/screens/SettingsScreen.tsx</v>
+        <v>src/screens/DeviceContactsScreen.tsx</v>
       </c>
       <c r="D124" t="str">
-        <v>BL-034 (Sprint 4): Added Backup and Restore buttons to Premium Features card. Hidden file input for restore. Success reloads page after 1.2s. Error feedback clears after 3s.</v>
+        <v>BL-030: מסך ייבוא מהטלפון — תהליך consent/permission/list/import; dedup טלפון; fallback ל-web; @capacitor-community/contacts</v>
       </c>
       <c r="E124" t="str">
         <v>feature</v>
@@ -3380,19 +3392,19 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>2026-04-29</v>
+        <v>2026-04-28</v>
       </c>
       <c r="B125" t="str">
-        <v>01:45</v>
+        <v>22:00</v>
       </c>
       <c r="C125" t="str">
-        <v>src/screens/ContactFormScreen.tsx</v>
+        <v>src/App.tsx</v>
       </c>
       <c r="D125" t="str">
-        <v>BL-035 (Sprint 4): Duplicate contact detection on new contact creation. findDuplicate() checks exact name match or phone (7+ digits stripped). Modal warns with matching name and offers "Save Anyway" or "Cancel". Edit mode excluded.</v>
+        <v>BL-030: נוסף lazy import ל-DeviceContactsScreen; נוסף route /device-contacts עם Premium gate</v>
       </c>
       <c r="E125" t="str">
-        <v>feature</v>
+        <v>improvement</v>
       </c>
       <c r="F125" t="str">
         <v>code_change</v>
@@ -3406,33 +3418,683 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B126" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C126" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D126" t="str">
+        <v>BL-030: נוסף כרטיס קיצור דרך «ייבוא מהטלפון» בראש מסך Import — מנווט ל-/device-contacts</v>
+      </c>
+      <c r="E126" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F126" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G126" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H126" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B127" t="str">
+        <v>22:00</v>
+      </c>
+      <c r="C127" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Sprint 3 מסומן כ-✅ COMPLETE; BL-024/025/027/028/029 הועברו ל-Sprint 4</v>
+      </c>
+      <c r="E127" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F127" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G127" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H127" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B128" t="str">
+        <v>23:00</v>
+      </c>
+      <c r="C128" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D128" t="str">
+        <v>BUG-043: תוקן — חגים רב-יומיים הציגו נקודה רק ביום הראשון; getHolidaysForDay עודכן לבדיקת טווח [date, endDate]; רשימת חודש מסוננת לפי חפיפה עם החודש הנוכחי; isSameMonth הוסר מה-imports</v>
+      </c>
+      <c r="E128" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F128" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G128" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H128" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B129" t="str">
+        <v>23:00</v>
+      </c>
+      <c r="C129" t="str">
+        <v>src/data/holidays.ts</v>
+      </c>
+      <c r="D129" t="str">
+        <v>BUG-044: נוסף sukkot-2026 (15-22 תשרי תשפ״ז, 25 ספטמבר–2 אוקטובר 2026) — ה-entry של 2025 קיים אך 2026 חסר</v>
+      </c>
+      <c r="E129" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F129" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G129" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H129" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B130" t="str">
+        <v>23:30</v>
+      </c>
+      <c r="C130" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D130" t="str">
+        <v>BL-045: שיפור celebration feedback — צליל: C5/E5/G5 אקורד גדול arpeggio במקום oscillator; אנימציה: 10 חלקיקים (במקום 6), גדולים יותר (text-xl), פיזור רחב יותר (±85px/±110px), 1.6s</v>
+      </c>
+      <c r="E130" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F130" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G130" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H130" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="B131" t="str">
+        <v>23:30</v>
+      </c>
+      <c r="C131" t="str">
+        <v>src/index.css</v>
+      </c>
+      <c r="D131" t="str">
+        <v>BL-045: keyframe particleBurst עודכן — scale-pop (0.4→1.6→0) + מסלול רחב יותר; אנימציה עודכנה ל-1.4s</v>
+      </c>
+      <c r="E131" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F131" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G131" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H131" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
         <v>2026-04-29</v>
       </c>
-      <c r="B126" t="str">
-        <v>01:45</v>
-      </c>
-      <c r="C126" t="str">
+      <c r="B132" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C132" t="str">
+        <v>src/services/exportService.ts</v>
+      </c>
+      <c r="D132" t="str">
+        <v>BL-025: exportContactsToCSV — ייצוא כל שדות קשר ל-CSV עם BOM לתמיכה ב-Excel Hebrew; PapaParse</v>
+      </c>
+      <c r="E132" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F132" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G132" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H132" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B133" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C133" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D133" t="str">
+        <v>BL-025: נוסף כפתור ייצוא CSV בכרטיס Premium Features; exportDone state עם הצלחה feedback 2.5s</v>
+      </c>
+      <c r="E133" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F133" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G133" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H133" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B134" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C134" t="str">
         <v>src/i18n/index.ts</v>
       </c>
-      <c r="D126" t="str">
-        <v>BL-024+034+035: Added 13 i18n keys in EN+HE: settings_backupData/Success, settings_restoreData/Success/Error, contactForm_duplicateTitle/Body/SaveAnyway.</v>
-      </c>
-      <c r="E126" t="str">
+      <c r="D134" t="str">
+        <v>BL-025: נוספו מפתחות settings_exportContacts + settings_exportSuccess ב-EN+HE</v>
+      </c>
+      <c r="E134" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F134" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G134" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H134" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B135" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C135" t="str">
+        <v>src/components/Navigation.tsx</v>
+      </c>
+      <c r="D135" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתור חזרה ב-PageHeader עודכן ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E135" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F135" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G135" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H135" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B136" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C136" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D136" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתור מחיקה ב-PageHeader עודכן ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E136" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F136" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G136" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H136" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B137" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C137" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D137" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתורי Edit/Delete בכרטיסי קבוצה עודכנו ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E137" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F137" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G137" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H137" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B138" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C138" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D138" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתורי Regenerate/Copy עודכנו ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E138" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F138" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G138" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H138" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B139" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C139" t="str">
+        <v>src/components/ui/Modal.tsx</v>
+      </c>
+      <c r="D139" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתור סגירה ב-Modal עודכן ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E139" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F139" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G139" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H139" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B140" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C140" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D140" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתור עריכה ב-PageHeader עודכן ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E140" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F140" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G140" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H140" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B141" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C141" t="str">
+        <v>src/screens/HolidayDetailScreen.tsx</v>
+      </c>
+      <c r="D141" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתור העתקת ברכה עודכן ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E141" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F141" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G141" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H141" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B142" t="str">
+        <v>00:30</v>
+      </c>
+      <c r="C142" t="str">
+        <v>src/screens/premium/BirthdayGreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D142" t="str">
+        <v>BL-029 WCAG 2.5.5: כפתורי Regenerate/Copy עודכנו ל-min-w/h-[48px] flex items-center justify-center</v>
+      </c>
+      <c r="E142" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F142" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G142" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H142" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B143" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C143" t="str">
+        <v>src/services/hapticService.ts</v>
+      </c>
+      <c r="D143" t="str">
+        <v>BL-024 (Sprint 4): שירות haptic feedback — hapticLight/Medium/Success/Error; Capacitor.isNativePlatform() guard; graceful no-op בדפדפן</v>
+      </c>
+      <c r="E143" t="str">
         <v>feature</v>
       </c>
-      <c r="F126" t="str">
-        <v>code_change</v>
-      </c>
-      <c r="G126" t="str">
-        <v>Agent 1</v>
-      </c>
-      <c r="H126" t="str">
+      <c r="F143" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G143" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H143" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B144" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C144" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D144" t="str">
+        <v>BL-024: hapticSuccess() מופעל לאחר שמירת איש קשר; BL-035: findDuplicate() + Modal אזהרה לשם/טלפון כפול + doSave() refactor</v>
+      </c>
+      <c r="E144" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F144" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G144" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H144" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B145" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C145" t="str">
+        <v>src/components/ChannelPicker.tsx</v>
+      </c>
+      <c r="D145" t="str">
+        <v>BL-024: hapticMedium() מופעל עם שליחת ברכה בכל ערוץ</v>
+      </c>
+      <c r="E145" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F145" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G145" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H145" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B146" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C146" t="str">
+        <v>src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D146" t="str">
+        <v>BL-024: hapticSuccess() בהפעלת קופון; hapticError() בכישלון</v>
+      </c>
+      <c r="E146" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F146" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G146" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H146" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B147" t="str">
+        <v>01:30</v>
+      </c>
+      <c r="C147" t="str">
+        <v>src/services/storageService.ts</v>
+      </c>
+      <c r="D147" t="str">
+        <v>BL-034 (Sprint 4): exportBackupJSON() ו-importBackupJSON() — מייצאים/מייבאים contacts+groups+drafts+settings כ-JSON עם version+timestamp</v>
+      </c>
+      <c r="E147" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F147" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G147" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H147" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B148" t="str">
+        <v>01:30</v>
+      </c>
+      <c r="C148" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D148" t="str">
+        <v>BL-034: כפתורי Backup/Restore בכרטיס Premium Features; hidden file input; feedback states</v>
+      </c>
+      <c r="E148" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F148" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G148" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H148" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B149" t="str">
+        <v>01:30</v>
+      </c>
+      <c r="C149" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D149" t="str">
+        <v>BL-024+034+035: מפתחות backup/restore/duplicate ב-EN+HE; 13 מפתחות חדשים סה"כ</v>
+      </c>
+      <c r="E149" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F149" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G149" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H149" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B150" t="str">
+        <v>02:00</v>
+      </c>
+      <c r="C150" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D150" t="str">
+        <v>Sprint 4 BL-024/025/027/028/029/034/035 מסומנים ✅ Done; BL-031/032/033/036/037/038 הועברו ל-Sprint 5; נוספו BL-046 עד BL-052 (7 משימות חדשות מהמשתמש: Import entry point, CSV label, device contacts visibility, BottomNav active tab, group assignment, Excel template, smart holiday suggestions by group purpose)</v>
+      </c>
+      <c r="E150" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F150" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G150" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H150" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B151" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="C151" t="str">
+        <v>scripts/make-changelog.js</v>
+      </c>
+      <c r="D151" t="str">
+        <v>שיפור מעקב changelog: הסקריפט מחדש קורא ישירות מ-changelog_queue.json במקום מערך hardcoded; 64 שורות legacy נשמרות כ-LEGACY_ROWS; כל השינויים העתידיים נרשמים אוטומטית; 24 רשומות שהיו חסרות שוחזרו — סה"כ 149 רשומות (היה 125)</v>
+      </c>
+      <c r="E151" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F151" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G151" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H151" t="str">
         <v>done</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H126"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H151"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 5: Import UX (BL-046/047/048), active tab (BL-049), group purpose & holiday suggestions (BL-052)
- BL-046: Import entry point in ContactsScreen header + empty-state shortcut (premium)
- BL-047: Restrict import to CSV-only; add 📄 CSV badge and i18n label
- BL-048: Device contacts CTA as prominent blue gradient card with divider
- BL-049: BottomNav active tab — dot indicator, larger icon (22px), bold primary-color label
- BL-052: GroupPurpose type + purpose selector pills + SUGGESTED_BASES holiday auto-suggestions in GroupsScreen

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H157"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -4092,9 +4092,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B152" t="str">
+        <v>04:00</v>
+      </c>
+      <c r="C152" t="str">
+        <v>src/screens/ContactsScreen.tsx</v>
+      </c>
+      <c r="D152" t="str">
+        <v>BL-046 Sprint 5: נוסף כפתור Import (FileUp) בכותרת לפרמיום; קיצור דרך ייבוא בEmpty State לפרמיום</v>
+      </c>
+      <c r="E152" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F152" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G152" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H152" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B153" t="str">
+        <v>04:00</v>
+      </c>
+      <c r="C153" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D153" t="str">
+        <v>BL-047: accept='.csv,.xlsx' → accept='.csv'; תווית CSV-only בולטת עם badge. BL-048: כפתור device contacts עוצב כ-CTA כחול בולט עם gradient+shadow; מפריד 'או העלה קובץ CSV'</v>
+      </c>
+      <c r="E153" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F153" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G153" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H153" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B154" t="str">
+        <v>04:00</v>
+      </c>
+      <c r="C154" t="str">
+        <v>src/components/Navigation.tsx</v>
+      </c>
+      <c r="D154" t="str">
+        <v>BL-049: שיפור Active tab — icon גדול יותר (22px), label בצבע primary עם fontWeight 800, נקודת אינדיקטור קטנה מתחת ל-label</v>
+      </c>
+      <c r="E154" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F154" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G154" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H154" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B155" t="str">
+        <v>04:30</v>
+      </c>
+      <c r="C155" t="str">
+        <v>src/types/index.ts</v>
+      </c>
+      <c r="D155" t="str">
+        <v>BL-052: GroupPurpose union type (family/friends/work/clients/hr/community/custom) + purpose?: GroupPurpose שדה ב-Group interface</v>
+      </c>
+      <c r="E155" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F155" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G155" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H155" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B156" t="str">
+        <v>04:30</v>
+      </c>
+      <c r="C156" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D156" t="str">
+        <v>BL-052: SUGGESTED_BASES lookup לפי purpose; applyPurpose() מוסיף הצעות ל-selectedHolidayIds ללא דריסה; purpose selector pills במודל; ✦ badge על חגים מוצעים ברשימה; form+save+openForm מעודכנים עם purpose</v>
+      </c>
+      <c r="E156" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F156" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G156" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H156" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B157" t="str">
+        <v>04:30</v>
+      </c>
+      <c r="C157" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D157" t="str">
+        <v>BL-046/047/048/049/052: נוספו 20 מפתחות ב-EN+HE: import_csvOnly/fromPhoneDesc/orCSV; group_purpose/hint + 7 purpose labels; group_holidays_selected</v>
+      </c>
+      <c r="E157" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F157" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G157" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H157" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H151"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H157"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sprint 5: Group assignment on import (BL-050), CSV template download (BL-051)
- BL-050: Group selector in import done-step; assign all imported contacts to a group via updateGroup; Set merge prevents duplicates; success feedback shows group name
- BL-051: downloadCSVTemplate() generates CSV with BOM, Hebrew headers, and sample row; purple download button in upload step

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H160"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -4248,9 +4248,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B158" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C158" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D158" t="str">
+        <v>BL-050: group assignment UI בשלב done — select + כפתור assign; מיזוג contactIds עם Set למניעת כפילויות; groupAssigned feedback</v>
+      </c>
+      <c r="E158" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F158" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G158" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H158" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B159" t="str">
+        <v>12:01</v>
+      </c>
+      <c r="C159" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D159" t="str">
+        <v>BL-051: downloadCSVTemplate() — Blob CSV עם BOM + כותרות עבריות + שורת דוגמה; כפתור הורדה בשלב upload</v>
+      </c>
+      <c r="E159" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F159" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G159" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H159" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B160" t="str">
+        <v>12:02</v>
+      </c>
+      <c r="C160" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D160" t="str">
+        <v>BL-050/051: נוספו 10 מפתחות EN+HE: import_addToGroup/Hint/selectGroup/assignGroup/groupAssigned/noGroups/downloadTemplate/templateHint</v>
+      </c>
+      <c r="E160" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F160" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G160" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H160" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H157"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H160"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add BL-059 Premium holiday reminder notifications (Sprint 9)
- BACKLOG.md: BL-059 added to Sprint 4+ Future table
- BACKLOG.csv: BL-059 row appended (ID unique, sequential after BL-058)
- FEATURES.md: feature described in Sprint 9 Planned section;
  Free vs Premium comparison table added to Upgrade screen docs;
  BL-032 moved to Sprint 9 section, BL-033 to Sprint 10 section
- changelog.xlsx: 187 entries (3 new doc entries)
- No implementation started; Sprint 8 unchanged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H188"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -4976,9 +4976,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B186" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="C186" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D186" t="str">
+        <v>BL-059 נוסף: Premium holiday reminder notifications — Sprint 9; Push/SMS/Email/WhatsApp; dedup; Premium gate</v>
+      </c>
+      <c r="E186" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F186" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G186" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H186" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B187" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="C187" t="str">
+        <v>BACKLOG.csv</v>
+      </c>
+      <c r="D187" t="str">
+        <v>BL-059 שורה חדשה ב-BACKLOG.csv — Premium holiday reminder notifications</v>
+      </c>
+      <c r="E187" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F187" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G187" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H187" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B188" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="C188" t="str">
+        <v>FEATURES.md</v>
+      </c>
+      <c r="D188" t="str">
+        <v>BL-059 תועד ב-FEATURES.md: תיאור Feature, Sprint 9 Planned section, טבלת Free vs Premium עודכנה עם Holiday reminders + Notification channels</v>
+      </c>
+      <c r="E188" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F188" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G188" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H188" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H185"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H188"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BL-062): generic upgrade CTA text + clearer Hebrew hero title
BUG-045: CTA button was using provider-specific text (payme_goPayMe →
'שלם עם PayMe'). Added generic upgrade_cta key (EN: 'Upgrade Now' /
HE: 'שדרג עכשיו') and replaced the button text in UpgradeScreen.

BUG-046: upgrade_unlockEverything HE was 'פתח הכל' (vague). Changed
to 'שדרג לפרמיום' (Upgrade to Premium) — clearly communicates intent.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H195"/>
+  <dimension ref="A1:H198"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -5236,9 +5236,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B196" t="str">
+        <v>16:10</v>
+      </c>
+      <c r="C196" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D196" t="str">
+        <v>BUG-045/BL-062: נוסף מפתח upgrade_cta גנרי (EN: 'Upgrade Now' / HE: 'שדרג עכשיו') — ללא שם ספק; תוקן upgrade_unlockEverything בעברית מ-'פתח הכל' ל-'שדרג לפרמיום' (BUG-046)</v>
+      </c>
+      <c r="E196" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F196" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G196" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H196" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B197" t="str">
+        <v>16:10</v>
+      </c>
+      <c r="C197" t="str">
+        <v>src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D197" t="str">
+        <v>BUG-045/BL-062: הוחלף t('payme_goPayMe') ב-t('upgrade_cta') בכפתור ה-CTA הראשי — הטקסט עכשיו גנרי ללא שם ספק</v>
+      </c>
+      <c r="E197" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F197" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G197" t="str">
+        <v>Agent 1</v>
+      </c>
+      <c r="H197" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B198" t="str">
+        <v>16:11</v>
+      </c>
+      <c r="C198" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D198" t="str">
+        <v>BUG-045 ו-BUG-046: תועדו שני באגים בדף השדרוג — טקסט CTA ספציפי לספק ו-כותרת גיבור לא ברורה; שניהם סומנו כתוקנו</v>
+      </c>
+      <c r="E198" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F198" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G198" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H198" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H195"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H198"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(BL-063): log greeting type + Hebrew grammar bugs for Sprint 11
BUG-047: Switching VIP/Professional/Casual tier updates tone state but
does not auto-regenerate the displayed message. Root cause: no reactive
path re-invokes generate() on tone change.

BUG-048: Hebrew 'friendly' generic body templates contain unnatural
phrasing (e.g. "לברר מה שלומך" — wrong verb). Templates need review
against native-speaker examples.

Both tracked in BL-063, planned for Sprint 11. No code changes.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H200"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -5314,9 +5314,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B199" t="str">
+        <v>16:22</v>
+      </c>
+      <c r="C199" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D199" t="str">
+        <v>BL-063: נוסף תיאור מלא לבאג — סוג ברכה לא מיושם (אין רגנרציה אוטומטית) + דקדוק עברי שגוי בתבניות; מתוכנן לספרינט 11</v>
+      </c>
+      <c r="E199" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F199" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G199" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H199" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="B200" t="str">
+        <v>16:22</v>
+      </c>
+      <c r="C200" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D200" t="str">
+        <v>BUG-047 (סוג ברכה לא מיושם) ו-BUG-048 (דקדוק עברי שגוי): תועדו שני באגים חדשים; שניהם פתוחים ומתוכננים לספרינט 11</v>
+      </c>
+      <c r="E200" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F200" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G200" t="str">
+        <v>Agent 4</v>
+      </c>
+      <c r="H200" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H198"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H200"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-051, BUG-052): remove duplicate upgrade CTA + commit PaymeScreen demo mode
BUG-051: UpgradeScreen had two identical CTA buttons (upgrade_cta/CreditCard
and upgrade_now/Crown). Removed the older upgrade_cta block; only the
Crown/upgrade_now button above the coupon section remains. Removed unused
CreditCard import.

BUG-052: PaymeScreen demo-mode rewrite (BUG-049) existed only in working
directory and was never committed. Committed now — screen shows amber demo
notice (payme_demoNotice) + activate button (payme_activateDemo) with no
form or createPaymentLink.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H232"/>
+  <dimension ref="A1:H235"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6198,9 +6198,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B233" t="str">
+        <v>11:30</v>
+      </c>
+      <c r="C233" t="str">
+        <v>src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D233" t="str">
+        <v>תוקן BUG-051 — הוסר כפתור upgrade_cta/CreditCard הכפול; נשמר רק כפתור upgrade_now/Crown מעל חלק הקופון; הוסר import של CreditCard שלא בשימוש</v>
+      </c>
+      <c r="E233" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F233" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G233" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H233" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B234" t="str">
+        <v>11:30</v>
+      </c>
+      <c r="C234" t="str">
+        <v>src/screens/PaymeScreen.tsx</v>
+      </c>
+      <c r="D234" t="str">
+        <v>תוקן BUG-052 — שינויי מצב הדגמה של PaymeScreen לא הועלו ל-git; הועלה הגרסה הנכונה: מסך הדגמה עם payme_demoNotice ו-payme_activateDemo ללא form/createPaymentLink</v>
+      </c>
+      <c r="E234" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F234" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G234" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H234" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B235" t="str">
+        <v>11:31</v>
+      </c>
+      <c r="C235" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D235" t="str">
+        <v>נוספו BUG-051 ו-BUG-052 — כפתור CTA כפול ב-UpgradeScreen וגרסת PaymeScreen שלא הועלתה; שניהם סומנו כ-fixed</v>
+      </c>
+      <c r="E235" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F235" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G235" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H235" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H232"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H235"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-053, BUG-054): date picker RTL fix + Gematria day dropdown
BUG-053: Date inputs (lastContactDate, birthday) had type="date" but no
dir="ltr". In RTL documents the browser suppresses the native calendar
picker; adding dir="ltr" restores it on both desktop and mobile.

BUG-054: Hebrew birthday day options already used gematriya() but all Bug
Fix 1 changes (gematriya label, formatHebrewBirthdayDisplay util, Hebrew
birthday row in ContactDetailScreen, BirthdayEntry type + RTL arrows in
CalendarScreen, QA test IDs T118-T120) were never staged or pushed.
Committing all of them now.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H235"/>
+  <dimension ref="A1:H241"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6276,9 +6276,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B236" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C236" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D236" t="str">
+        <v>תוקן BUG-053 — נוסף dir='ltr' לשני שדות תאריך (lastContactDate ו-birthday) כדי שלוח שנה ייפתח בלחיצה במצב RTL</v>
+      </c>
+      <c r="E236" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F236" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G236" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H236" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B237" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C237" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D237" t="str">
+        <v>תוקן BUG-054 — הועלו שינויי Bug Fix 1 שלא הועלו: gematriya(d) כתווית ביום עברי, import של gematriya</v>
+      </c>
+      <c r="E237" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F237" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G237" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H237" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B238" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C238" t="str">
+        <v>src/utils/hebrewDateUtils.ts</v>
+      </c>
+      <c r="D238" t="str">
+        <v>הועלה פונקציית formatHebrewBirthdayDisplay — ממיר DD-MM לפורמט 'כ״א בטבת'</v>
+      </c>
+      <c r="E238" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F238" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G238" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H238" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B239" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C239" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D239" t="str">
+        <v>הועלה שורת תצוגת יום הולדת עברי ב-ContactDetailScreen עם formatHebrewBirthdayDisplay</v>
+      </c>
+      <c r="E239" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F239" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G239" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H239" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B240" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C240" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D240" t="str">
+        <v>הועלו תיקוני Bug Fix 1: חצי ניווט RTL תקינים, סוג BirthdayEntry לאירועי יום הולדת עברי/גרגוריאני עצמאיים</v>
+      </c>
+      <c r="E240" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F240" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G240" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H240" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B241" t="str">
+        <v>12:01</v>
+      </c>
+      <c r="C241" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D241" t="str">
+        <v>נוספו BUG-053 ו-BUG-054 — שדות תאריך לא פותחים לוח שנה ב-RTL; יום עברי לא בגמטריה (שינויים לא הועלו); שניהם סומנו כ-fixed</v>
+      </c>
+      <c r="E241" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F241" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G241" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H241" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H235"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H241"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-055): improve date picker icon visibility in dark mode
- Added --calendar-picker-invert CSS variable to applyTheme (themes.ts):
  value '1' for isDark themes, '0' for light themes
- Added --calendar-picker-invert: 0 default to :root in index.css
- Styled ::-webkit-calendar-picker-indicator: 20x20px, opacity 0.65,
  filter: invert(var(--calendar-picker-invert)) for dark mode, hover shows
  var(--color-surface-2) background. No hardcoded colors.
- Works in all themes; RTL layout and value handling unchanged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H241"/>
+  <dimension ref="A1:H244"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6432,9 +6432,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B242" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C242" t="str">
+        <v>src/index.css</v>
+      </c>
+      <c r="D242" t="str">
+        <v>תוקן BUG-055 — נוספו עיצוב CSS ל-::-webkit-calendar-picker-indicator: גודל 20×20px, opacity 0.65, hover עם רקע var(--color-surface-2), filter: invert(var(--calendar-picker-invert)) לנראות בתמה כהה</v>
+      </c>
+      <c r="E242" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F242" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G242" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H242" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B243" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C243" t="str">
+        <v>src/data/themes.ts</v>
+      </c>
+      <c r="D243" t="str">
+        <v>נוספה משתנה CSS --calendar-picker-invert ב-applyTheme: '1' לתמות כהות (isDark), '0' לתמות בהירות</v>
+      </c>
+      <c r="E243" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F243" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G243" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H243" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B244" t="str">
+        <v>13:01</v>
+      </c>
+      <c r="C244" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D244" t="str">
+        <v>נוסף BUG-055 — אייקון לוח שנה לא גלוי בתמה כהה; סומן כ-fixed</v>
+      </c>
+      <c r="E244" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F244" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G244" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H244" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H241"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H244"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-056): open date picker on full field click via showPicker()
- Added lastContactRef and birthdayRef (useRef<HTMLInputElement>) to both
  date inputs in ContactFormScreen
- Added openDatePicker() helper: calls ref.current?.showPicker() with
  ref.current?.click() fallback; attached to onClick on both date inputs
- Added cursor: pointer to input[type="date"].form-input in index.css,
  consistent with existing select.form-input cursor style
- Date value/storage logic unchanged; RTL dir="ltr" unchanged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H244"/>
+  <dimension ref="A1:H247"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6510,9 +6510,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B245" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C245" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D245" t="str">
+        <v>תוקן BUG-056 — נוספו refs (lastContactRef, birthdayRef) ופונקציית openDatePicker עם showPicker()/click() לשדות תאריך; onClick על כל שדה פותח לוח שנה בלחיצה בכל מקום</v>
+      </c>
+      <c r="E245" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F245" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G245" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H245" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B246" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C246" t="str">
+        <v>src/index.css</v>
+      </c>
+      <c r="D246" t="str">
+        <v>נוסף cursor: pointer ל-input[type='date'].form-input בהתאם לסגנון select.form-input הקיים</v>
+      </c>
+      <c r="E246" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F246" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G246" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H246" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B247" t="str">
+        <v>14:01</v>
+      </c>
+      <c r="C247" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D247" t="str">
+        <v>נוסף BUG-056 — שדות תאריך לא פותחים לוח שנה בלחיצה על כל השדה; סומן כ-fixed</v>
+      </c>
+      <c r="E247" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F247" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G247" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H247" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H244"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H247"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-057): Hebrew birthday dropdowns clear on partial selection
Root cause: hbParts useMemo derived from form.hebrewBirthday, which is only
written when both day AND month are valid. Selecting one part while the
other was empty caused setHebBirthday to write undefined, making hbParts
return '' and resetting the dropdown to the placeholder immediately.

Fix: replaced useMemo hbParts with useState hbDay/hbMonth (initialized from
existing.hebrewBirthday). Dropdowns bind to local state so selections
persist visually regardless of whether the form has a complete value yet.
setHebBirthday logic unchanged — still only persists when both parts valid.
Clear button now also resets local state. Removed unused useMemo import.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H247"/>
+  <dimension ref="A1:H249"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6588,9 +6588,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B248" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C248" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D248" t="str">
+        <v>תוקן BUG-057 — דרופדאון יום הולדת עברי מאפסים לאחר בחירה: הוחלף useMemo של hbParts ב-useState של hbDay/hbMonth; ערך מקומי נשמר גם כשרק חלק אחד נבחר; כפתור ניקוי מאפס גם state מקומי</v>
+      </c>
+      <c r="E248" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F248" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G248" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H248" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B249" t="str">
+        <v>15:01</v>
+      </c>
+      <c r="C249" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D249" t="str">
+        <v>נוסף BUG-057 — דרופדאון יום הולדת עברי מתאפסים לאחר בחירה חלקית; סומן כ-fixed</v>
+      </c>
+      <c r="E249" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F249" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G249" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H249" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H247"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H249"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-058): Modal focus trap re-fires on every keystroke, stealing focus
Root cause: Modal useEffect had [isOpen, onClose] as deps. onClose is an
inline arrow function in callers (e.g. GroupsScreen) — new reference on
every render. Each form keystroke re-rendered GroupsScreen, creating a new
onClose reference, causing the Modal's useEffect to re-run and call
requestAnimationFrame(() => first?.focus()), which moved focus away from
the active input to the first focusable element in the modal.

Fix: added onCloseRef updated by a dedicated useEffect([onClose]). The
focus-trap effect now depends only on [isOpen] — runs only when the modal
opens or closes, never on prop reference churn. Escape key handler reads
onCloseRef.current (always the latest value). Affects all modals in app.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H249"/>
+  <dimension ref="A1:H251"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6640,9 +6640,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B250" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C250" t="str">
+        <v>src/components/ui/Modal.tsx</v>
+      </c>
+      <c r="D250" t="str">
+        <v>תוקן BUG-058 — שדה תיאור בטופס קבוצה מאבד פוקוס אחרי כל תו: הוסר onClose מ-dependency array של useEffect הראשי; הוחלף ב-onCloseRef שמתעדכן ב-useEffect נפרד. הפוקוס-טרפ מופעל רק בפתיחה/סגירה של המודאל</v>
+      </c>
+      <c r="E250" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F250" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G250" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H250" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>2026-04-30</v>
+      </c>
+      <c r="B251" t="str">
+        <v>16:01</v>
+      </c>
+      <c r="C251" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D251" t="str">
+        <v>נוסף BUG-058 — שדה תיאור בטופס קבוצה מאבד פוקוס; סומן כ-fixed</v>
+      </c>
+      <c r="E251" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F251" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G251" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H251" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H249"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H251"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refine prompt validation rule (skip low-impact prompts)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H256"/>
+  <dimension ref="A1:H257"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6822,9 +6822,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B257" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C257" t="str">
+        <v>CLAUDE.md</v>
+      </c>
+      <c r="D257" t="str">
+        <v>נוסף כלל אימות פרומפטים — validation נדרש לפיצ'רים/באגים/שיפורים ותכנון בלבד; דילוג על steering פשוט, UI קטן, הבהרות; פורמט דוח עם Prompt Type/Clarity/Risk/Issues/Recommendation</v>
+      </c>
+      <c r="E257" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F257" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G257" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H257" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H256"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H257"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Disable premium gates for MVP testing (TEMP_PREMIUM_UNLOCK)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H257"/>
+  <dimension ref="A1:H259"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6848,9 +6848,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B258" t="str">
+        <v>10:30</v>
+      </c>
+      <c r="C258" t="str">
+        <v>src/context/AppContext.tsx</v>
+      </c>
+      <c r="D258" t="str">
+        <v>TEMP BL-070: נוסף TEMP_PREMIUM_UNLOCK = true — כל שערי Premium מושבתים זמנית לצורך בדיקות MVP; שורה אחת להחזרה ל-false לפני פרודקשן</v>
+      </c>
+      <c r="E258" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F258" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G258" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H258" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B259" t="str">
+        <v>10:30</v>
+      </c>
+      <c r="C259" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D259" t="str">
+        <v>נוסף BL-070 — משימת תזכורת pre-launch: השבת TEMP_PREMIUM_UNLOCK לפני פרודקשן</v>
+      </c>
+      <c r="E259" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F259" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G259" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H259" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H257"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H259"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: RTL pricing bidi in Settings + timeline direction in WhatsNew
- SettingsScreen: replace hardcoded /mo with t('upgrade_month'), wrap
  price in dir=ltr to prevent RTL bidi reversal (BUG-062)
- WhatsNewScreen: timeline line/dot/padding now flip sides in RTL
  using isRTL flag from useLang() (BUG-063)
- BUG_REPORT.md: mark BUG-047 and BUG-048 as fixed (Sprint 11 drift)
- BACKLOG.md: BL-063 marked Done

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H259"/>
+  <dimension ref="A1:H263"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -6900,9 +6900,113 @@
         <v>done</v>
       </c>
     </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B260" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C260" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D260" t="str">
+        <v>תוקן BUG-062 — כפתור שדרוג בהגדרות הציג mo/₪29 ב-RTL; הוחלף /mo ב-t('upgrade_month') ועטוף ב-span dir=ltr</v>
+      </c>
+      <c r="E260" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F260" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G260" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H260" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B261" t="str">
+        <v>11:10</v>
+      </c>
+      <c r="C261" t="str">
+        <v>src/screens/WhatsNewScreen.tsx</v>
+      </c>
+      <c r="D261" t="str">
+        <v>תוקן BUG-063 — ציר זמן ב-WhatsNew היה בצד שמאל גם ב-RTL; נוסף isRTL flag; ציר, נקודה ו-padding מחליפים צד לפי כיוון שפה</v>
+      </c>
+      <c r="E261" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F261" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G261" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H261" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B262" t="str">
+        <v>11:15</v>
+      </c>
+      <c r="C262" t="str">
+        <v>BUG_REPORT.md</v>
+      </c>
+      <c r="D262" t="str">
+        <v>עודכן סטטוס BUG-047 ו-BUG-048 מ-open ל-fixed (תוקנו ב-Sprint 11 — תיעוד היה מאחור); נוספו BUG-062 ו-BUG-063</v>
+      </c>
+      <c r="E262" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F262" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G262" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H262" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B263" t="str">
+        <v>11:15</v>
+      </c>
+      <c r="C263" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D263" t="str">
+        <v>BL-063 סומן ✅ Done (היה 📋 Backlog בטעות — תוקן ב-Sprint 11)</v>
+      </c>
+      <c r="E263" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F263" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G263" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H263" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H259"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H263"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: RTL toggle switch direction in Settings and HolidayReminders
Toggle dot used left-0.5 + translateX(20px) regardless of language,
making OFF/ON visually reversed in Hebrew. Now uses right-0.5 and
translateX(-20px) when lang==='he'. (BUG-064)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H263"/>
+  <dimension ref="A1:H265"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7004,9 +7004,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B264" t="str">
+        <v>11:30</v>
+      </c>
+      <c r="C264" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D264" t="str">
+        <v>תוקן BUG-064 — נקודת toggle התחילה תמיד בשמאל גם ב-RTL; עדכון ל-right-0.5 + translateX(-20px) בעברית</v>
+      </c>
+      <c r="E264" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F264" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G264" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H264" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B265" t="str">
+        <v>11:30</v>
+      </c>
+      <c r="C265" t="str">
+        <v>src/screens/HolidayRemindersScreen.tsx</v>
+      </c>
+      <c r="D265" t="str">
+        <v>תוקן BUG-064 — 2 toggles (enabled + channels) תוקנו ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E265" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F265" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G265" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H265" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H263"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H265"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-065,BUG-066): RTL margin direction and i18n testimonials
BUG-065: Replace physical ml-1/ml-2 sibling-gap classes with logical
ms-1/ms-2 (margin-inline-start) in UpgradeScreen, CalendarScreen, and
GreetingEditorScreen so gaps render on the correct side in RTL.

BUG-066: Move UpgradeScreen testimonials from hardcoded English strings
to i18n keys with Hebrew translations in both EN and HE locales.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H265"/>
+  <dimension ref="A1:H270"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7056,9 +7056,139 @@
         <v>done</v>
       </c>
     </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B266" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C266" t="str">
+        <v>src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D266" t="str">
+        <v>תוקן BUG-065 — ml-1 הוחלף ב-ms-1 (margin-inline-start) כדי שהרווח יהיה בצד הנכון ב-RTL</v>
+      </c>
+      <c r="E266" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F266" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G266" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H266" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B267" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C267" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D267" t="str">
+        <v>תוקן BUG-065 — שני ml-2 בכותרות קטגוריות הוחלפו ב-ms-2 כדי שספירת הפריטים תופיע בצד הנכון ב-RTL</v>
+      </c>
+      <c r="E267" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F267" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G267" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H267" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B268" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C268" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D268" t="str">
+        <v>תוקן BUG-065 — ml-1 בסרגל הצעות AI הוחלף ב-ms-1</v>
+      </c>
+      <c r="E268" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F268" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G268" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H268" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B269" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C269" t="str">
+        <v>src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D269" t="str">
+        <v>תוקן BUG-066 — המלצות המשתמשים (testimonials) היו hardcoded באנגלית; הועברו למפתחות i18n עם תרגום לעברית</v>
+      </c>
+      <c r="E269" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F269" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G269" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H269" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B270" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C270" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D270" t="str">
+        <v>נוספו 6 מפתחות i18n לעדויות משתמשים ב-UpgradeScreen (upgrade_testimonial_1/2_name/role/quote) — EN + HE</v>
+      </c>
+      <c r="E270" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F270" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G270" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H270" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H265"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H270"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-067): Flip decorative borderLeft accent bars to borderRight in RTL
Six screens used physical borderLeft for card accent styling. In RTL
these bars appeared on the wrong (end) side. Fixed with a computed
property key [lang === 'he' ? 'borderRight' : 'borderLeft'] on each.

Added useLang import + const { lang } = useLang() to DashboardScreen,
GreetingEditorScreen, and ContactFormScreen which lacked it.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H270"/>
+  <dimension ref="A1:H276"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7186,9 +7186,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B271" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C271" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D271" t="str">
+        <v>תוקן BUG-067 — borderLeft של כרטיסי ימי הולדת עבר לצד הנכון ב-RTL באמצעות computed property key</v>
+      </c>
+      <c r="E271" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F271" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G271" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H271" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B272" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C272" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D272" t="str">
+        <v>תוקן BUG-067 — borderLeft של כרטיסי התראות חגים עבר ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E272" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F272" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G272" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H272" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B273" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C273" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D273" t="str">
+        <v>תוקן BUG-067 — borderLeft של בלוק ציטוט חג עבר ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E273" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F273" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G273" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H273" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B274" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C274" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D274" t="str">
+        <v>תוקן BUG-067 — borderLeft של קטע שדות Premium עבר ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E274" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F274" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G274" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H274" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B275" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C275" t="str">
+        <v>src/screens/HolidayDetailScreen.tsx</v>
+      </c>
+      <c r="D275" t="str">
+        <v>תוקן BUG-067 — borderLeft של הערות רגישות עבר ל-RTL</v>
+      </c>
+      <c r="E275" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F275" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G275" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H275" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B276" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C276" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D276" t="str">
+        <v>תוקן BUG-067 — borderLeft של כרטיסי קבוצות עבר ל-RTL</v>
+      </c>
+      <c r="E276" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F276" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G276" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H276" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H270"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H276"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-068): Replace physical text-left/border-l-2 with logical RTL equivalents
All text-left class usages that represent "start" alignment replaced with
text-start (text-align: start) so text flows to the right in Hebrew RTL
instead of being forced left. Affects GroupsScreen (3), DashboardScreen (3),
SettingsScreen (5+border-s-2 accent), ImportContactsScreen (1 table header).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H276"/>
+  <dimension ref="A1:H280"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7342,9 +7342,113 @@
         <v>done</v>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B277" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C277" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D277" t="str">
+        <v>תוקן BUG-068 — text-left הוחלף ב-text-start (3 מופעים) כדי שהיישור יעקוב אחרי כיוון הטקסט</v>
+      </c>
+      <c r="E277" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F277" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G277" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H277" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B278" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C278" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D278" t="str">
+        <v>תוקן BUG-068 — text-left הוחלף ב-text-start (3 מופעים)</v>
+      </c>
+      <c r="E278" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F278" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G278" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H278" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B279" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C279" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D279" t="str">
+        <v>תוקן BUG-068 — text-left הוחלף ב-text-start (5 מופעים); border-l-2 הוחלף ב-border-s-2 בהדגשת אזור הסכנה</v>
+      </c>
+      <c r="E279" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F279" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G279" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H279" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B280" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C280" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D280" t="str">
+        <v>תוקן BUG-068 — text-left בכותרות טבלת CSV הוחלף ב-text-start</v>
+      </c>
+      <c r="E280" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F280" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G280" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H280" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H276"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H280"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-069): Flip ChevronRight disclosure/continue icons in RTL
In RTL flex layout ChevronRight appears on the left side of content
pointing rightward — the backward direction for RTL. Fixed by conditionally
rendering ChevronLeft when lang === 'he'. Affects SettingsScreen (5 list
item disclosure arrows) and OnboardingScreen (continue button).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H280"/>
+  <dimension ref="A1:H282"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7446,9 +7446,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B281" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C281" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D281" t="str">
+        <v>תוקן BUG-069 — 5 סמלי ChevronRight בפריטי רשימה עטופו בתנאי RTL (ChevronLeft בעברית); נוסף ייבוא ChevronLeft</v>
+      </c>
+      <c r="E281" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F281" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G281" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H281" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B282" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C282" t="str">
+        <v>src/screens/OnboardingScreen.tsx</v>
+      </c>
+      <c r="D282" t="str">
+        <v>תוקן BUG-069 — ChevronRight בכפתור המשך עבר ל-ChevronLeft בעברית; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E282" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F282" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G282" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H282" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H280"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H282"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-070): RTL physical CSS fixes in shared components
ContactCard: text-left → text-start, borderLeft urgency bar flips in RTL.
HolidayCard (compact): borderLeft accent flips in RTL.
Card: accent prop borderLeft flips in RTL — fixes every Card with accent prop.
ChannelPicker: text-left → text-start on label spans.
Added useLang import to ContactCard, HolidayCard, Card.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H282"/>
+  <dimension ref="A1:H286"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7498,9 +7498,113 @@
         <v>done</v>
       </c>
     </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B283" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C283" t="str">
+        <v>src/components/ContactCard.tsx</v>
+      </c>
+      <c r="D283" t="str">
+        <v>תוקן BUG-070 — text-left → text-start; borderLeft של פס דחיפות עבר ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E283" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F283" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G283" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H283" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B284" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C284" t="str">
+        <v>src/components/HolidayCard.tsx</v>
+      </c>
+      <c r="D284" t="str">
+        <v>תוקן BUG-070 — borderLeft של כרטיס חג מהיר עבר ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E284" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F284" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G284" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H284" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B285" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C285" t="str">
+        <v>src/components/ui/Card.tsx</v>
+      </c>
+      <c r="D285" t="str">
+        <v>תוקן BUG-070 — prop accent: borderLeft עבר ל-RTL; נוסף ייבוא useLang</v>
+      </c>
+      <c r="E285" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F285" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G285" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H285" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B286" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C286" t="str">
+        <v>src/components/ChannelPicker.tsx</v>
+      </c>
+      <c r="D286" t="str">
+        <v>תוקן BUG-070 — text-left → text-start על ספן תוויות הערוצים</v>
+      </c>
+      <c r="E286" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F286" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G286" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H286" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H282"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H286"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-071): i18n BirthdayGreetingEditorScreen hardcoded strings
Add 14 i18n keys (birthday_greeting_*, birthday_tier_*) in EN + HE.
Move BIRTHDAY_TIERS inside the component to use t() for label/desc.
Replace 8 hardcoded English strings with t() calls (subtitle, prompt,
style selector, tier names, preview labels, character count).
Fix CalendarScreen filter button to use t('calendar_filterByReligion')
for aria-label instead of hardcoded English.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H286"/>
+  <dimension ref="A1:H289"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7602,9 +7602,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B287" t="str">
+        <v>14:30</v>
+      </c>
+      <c r="C287" t="str">
+        <v>src/screens/premium/BirthdayGreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D287" t="str">
+        <v>תוקן BUG-071 — כל המחרוזות האנגליות hardcoded הועברו למפתחות i18n (כותרת, סגנונות, תצוגה מקדימה, ספירת תווים)</v>
+      </c>
+      <c r="E287" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F287" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G287" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H287" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B288" t="str">
+        <v>14:30</v>
+      </c>
+      <c r="C288" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D288" t="str">
+        <v>נוספו 14 מפתחות i18n לעורך ברכות יום הולדת (birthday_greeting_* + birthday_tier_*) — EN + HE</v>
+      </c>
+      <c r="E288" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F288" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G288" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H288" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B289" t="str">
+        <v>14:30</v>
+      </c>
+      <c r="C289" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D289" t="str">
+        <v>תוקן BUG-071 — aria-label של כפתור הסינון הוחלף ב-t('calendar_filterByReligion') במקום מחרוזת hardcoded</v>
+      </c>
+      <c r="E289" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F289" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G289" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H289" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H286"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H289"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-072): i18n ImportContactsScreen hardcoded strings
Add 13 i18n keys (import_field_*, import_stat_*) in EN + HE.
Move CONTACT_FIELDS inside main component to use t() for labels.
Add useT() to StepIndicator to use existing upload/map/done keys.
Replace hardcoded "Imported"/"Skipped"/"Total rows" stats with t().

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H289"/>
+  <dimension ref="A1:H291"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7680,9 +7680,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B290" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C290" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D290" t="str">
+        <v>תוקן BUG-072 — CONTACT_FIELDS הועבר לתוך הקומפוננטה עם t(); StepIndicator קיבל useT(); תוויות סטטיסטיקה הוחלפו ב-t()</v>
+      </c>
+      <c r="E290" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F290" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G290" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H290" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B291" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C291" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D291" t="str">
+        <v>נוספו 13 מפתחות i18n לייבוא אנשי קשר (import_field_* + import_stat_*) — EN + HE</v>
+      </c>
+      <c r="E291" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F291" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G291" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H291" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H289"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H291"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-073): Add missing aria-label to GroupsScreen edit/delete buttons
Icon-only Edit and Delete buttons on group cards lacked aria-label,
making them inaccessible to screen readers. Added t('groups_editGroup')
and t('groups_deleteGroup') using existing i18n keys.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H291"/>
+  <dimension ref="A1:H292"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7732,9 +7732,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B292" t="str">
+        <v>15:15</v>
+      </c>
+      <c r="C292" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D292" t="str">
+        <v>תוקן BUG-073 — כפתורי עריכה ומחיקה של קבוצות קיבלו aria-label לנגישות</v>
+      </c>
+      <c r="E292" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F292" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G292" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H292" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H291"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H292"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-074): Input icon positioning not RTL-aware
In Hebrew/RTL mode, leading/trailing icons in Input component appeared
on the wrong side with padding applied to the wrong edge. Added useLang
and isRTL flag to conditionally flip left-3/right-3 positioning and
pl-10/pr-10 padding based on text direction.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H292"/>
+  <dimension ref="A1:H293"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7758,9 +7758,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B293" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="C293" t="str">
+        <v>src/components/ui/Input.tsx</v>
+      </c>
+      <c r="D293" t="str">
+        <v>תיקון BUG-074: ממשק Input לא היה מודע ל-RTL — האייקונים הופיעו בצד הלא נכון בעברית. הוספת useLang ו-isRTL לניהול מיקום האייקון והריפוד בהתאם לכיוון הטקסט.</v>
+      </c>
+      <c r="E293" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F293" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G293" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H293" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H292"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H293"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-075): PrivacyScreen all content hardcoded in English
All 10 section titles/bodies plus hero title, badge, intro, footer were
locked to English strings in a module-level array. Added 25 i18n keys
(EN+HE) and moved SECTIONS inside the component to use t() so the full
privacy policy displays in Hebrew when language is set to HE.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H293"/>
+  <dimension ref="A1:H295"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7784,9 +7784,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B294" t="str">
+        <v>15:45</v>
+      </c>
+      <c r="C294" t="str">
+        <v>src/screens/PrivacyScreen.tsx</v>
+      </c>
+      <c r="D294" t="str">
+        <v>תיקון BUG-075: כל תוכן מסך הפרטיות היה קשיח באנגלית. הועבר מערך SECTIONS לתוך הקומפוננטה עם שימוש ב-t() לכל הכותרות ותוכן הסעיפים.</v>
+      </c>
+      <c r="E294" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F294" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G294" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H294" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B295" t="str">
+        <v>15:45</v>
+      </c>
+      <c r="C295" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D295" t="str">
+        <v>תיקון BUG-075: הוספת 25 מפתחות i18n חדשים (EN+HE) עבור מסך הפרטיות: privacy_hero_title, privacy_last_updated, privacy_badge, privacy_intro, privacy_footer, privacy_s1 עד privacy_s10 (כותרות וגוף טקסט).</v>
+      </c>
+      <c r="E295" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F295" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G295" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H295" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H293"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H295"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BUG-076): Replace remaining physical CSS margins with logical properties
ml-auto → ms-auto, ml-* → ms-*, mr-* → me-*, text-right → text-end
across BirthdayGreetingEditorScreen, App.tsx, DashboardScreen,
MediaAttachmentPicker, GreetingEditorScreen, and WhatsNewScreen.
Ensures correct RTL layout in Hebrew mode for all affected elements.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H295"/>
+  <dimension ref="A1:H301"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7836,9 +7836,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B296" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C296" t="str">
+        <v>src/screens/premium/BirthdayGreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D296" t="str">
+        <v>תיקון BUG-076: החלפת מחלקות CSS פיזיות (ml-*, mr-*, text-right) בתכונות לוגיות (ms-*, me-*, text-end) לתמיכה נכונה ב-RTL.</v>
+      </c>
+      <c r="E296" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F296" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G296" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H296" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B297" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C297" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="D297" t="str">
+        <v>תיקון BUG-076: החלפת מחלקות CSS פיזיות (ml-*, mr-*, text-right) בתכונות לוגיות (ms-*, me-*, text-end) לתמיכה נכונה ב-RTL.</v>
+      </c>
+      <c r="E297" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F297" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G297" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H297" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B298" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C298" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D298" t="str">
+        <v>תיקון BUG-076: החלפת מחלקות CSS פיזיות (ml-*, mr-*, text-right) בתכונות לוגיות (ms-*, me-*, text-end) לתמיכה נכונה ב-RTL.</v>
+      </c>
+      <c r="E298" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F298" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G298" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H298" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B299" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C299" t="str">
+        <v>src/components/MediaAttachmentPicker.tsx</v>
+      </c>
+      <c r="D299" t="str">
+        <v>תיקון BUG-076: החלפת מחלקות CSS פיזיות (ml-*, mr-*, text-right) בתכונות לוגיות (ms-*, me-*, text-end) לתמיכה נכונה ב-RTL.</v>
+      </c>
+      <c r="E299" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F299" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G299" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H299" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B300" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C300" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D300" t="str">
+        <v>תיקון BUG-076: החלפת מחלקות CSS פיזיות (ml-*, mr-*, text-right) בתכונות לוגיות (ms-*, me-*, text-end) לתמיכה נכונה ב-RTL.</v>
+      </c>
+      <c r="E300" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F300" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G300" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H300" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B301" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C301" t="str">
+        <v>src/screens/WhatsNewScreen.tsx</v>
+      </c>
+      <c r="D301" t="str">
+        <v>תיקון BUG-076: החלפת מחלקות CSS פיזיות (ml-*, mr-*, text-right) בתכונות לוגיות (ms-*, me-*, text-end) לתמיכה נכונה ב-RTL.</v>
+      </c>
+      <c r="E301" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F301" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G301" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H301" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H295"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H301"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: CalendarScreen mr-1 ml-1 → mx-1 on Hebrew birthday span
Minor cleanup — symmetric physical margins replaced with logical mx-1.
Completes the RTL physical CSS sweep (zero physical margin/alignment
classes remaining across all .tsx files).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H301"/>
+  <dimension ref="A1:H302"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -7992,9 +7992,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B302" t="str">
+        <v>16:10</v>
+      </c>
+      <c r="C302" t="str">
+        <v>src/screens/CalendarScreen.tsx</v>
+      </c>
+      <c r="D302" t="str">
+        <v>תיקון: החלפת mr-1 ml-1 (מרווחים פיזיים סימטריים) ב-mx-1 (מרווח אופקי לוגי) על span תאריך לידה עברי.</v>
+      </c>
+      <c r="E302" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F302" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G302" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H302" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H301"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H302"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(BL-064): one-tap greeting send — ChannelPicker in Quick Send panel + holiday CTAs
Quick Send panel now opens ChannelPicker (all channels: WhatsApp/SMS/Email/
Copy/Share) instead of direct WhatsApp, giving users full channel choice.

Today's and tomorrow's holiday highlight banners now include an inline
"Send Greeting" CTA that opens the Greeting Editor pre-filled with the holiday.

Also adds BL-075 to backlog: 3-dot overflow menu for contact edit/delete.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H310"/>
+  <dimension ref="A1:H312"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8226,9 +8226,61 @@
         <v>done</v>
       </c>
     </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B311" t="str">
+        <v>18:00</v>
+      </c>
+      <c r="C311" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D311" t="str">
+        <v>BL-064: ChannelPicker שולב ב-Quick Send Panel (מחליף כפתור WhatsApp ישיר); כפתור שלח ברכה נוסף לכרטיסי חג היום ומחר; ייבוא ChannelPicker וstate channelPickerData; הוסר openWhatsApp שאינו בשימוש</v>
+      </c>
+      <c r="E311" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F311" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G311" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H311" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B312" t="str">
+        <v>18:01</v>
+      </c>
+      <c r="C312" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D312" t="str">
+        <v>BL-064: 2 מפתחות i18n חדשים (EN+HE): dashboard_quick_send_channel, dashboard_send_greeting</v>
+      </c>
+      <c r="E312" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F312" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G312" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H312" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H310"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H312"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BL-077): exact-match mapping table + erev-adjust + 3 wrong match strings
Replace all startsWith matching with a strict controlled mapping table —
every hebcalName is the exact string @hebcal/core returns in Israel mode.

Fixes:
- simchat-torah: 'Simchat Torah' → 'Shmini Atzeret' (Israel mode combines them)
- shiva-asar-btammuz: 'Shiva Asar B\'Tammuz' → 'Tzom Tammuz' (Hebcal name)
- israel-independence-day: 'HaAtzma\'ut' → 'Yom HaAtzma\'ut' (full event name)

Add erevAdjust flag to restore Erev-based dates matching previous behavior:
affected holidays: Rosh Hashana, Yom Kippur, Sukkot, Passover, Shavuot, Simchat Torah.

Rosh Hashana uses hebcalYearSuffix to match 'Rosh Hashana 5786' exactly.

Validated: 21 before/after comparisons — zero date or endDate differences.
Build + lint clean.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H313"/>
+  <dimension ref="A1:H314"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8304,9 +8304,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B314" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="C314" t="str">
+        <v>src/data/holidays.ts</v>
+      </c>
+      <c r="D314" t="str">
+        <v>BL-077 תיקון: (1) 3 hebcalMatch שגויים תוקנו — simchat-torah: Shmini Atzeret, shiva-asar-btammuz: Tzom Tammuz, israel-independence-day: Yom HaAtzma'ut; (2) הוחלפה לוגיקת startsWith בטבלת mapping מבוקרת (exact match בלבד); (3) נוסף erevAdjust לשחזור תאריכי ערב (Rosh Hashana/Yom Kippur/Sukkot/Passover/Shavuot/Simchat Torah); (4) אומת: 21 השוואות BEFORE vs AFTER — אפס הבדלים</v>
+      </c>
+      <c r="E314" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F314" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G314" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H314" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H313"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H314"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(backlog): add BL-078 — mobile browser misleading message on device contacts import
UX improvement (Low priority): clarify "app required" vs "mobile required" messaging.
No implementation — backlog only.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H317"/>
+  <dimension ref="A1:H318"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8408,9 +8408,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B318" t="str">
+        <v>22:30</v>
+      </c>
+      <c r="C318" t="str">
+        <v>BACKLOG.md / BACKLOG.csv</v>
+      </c>
+      <c r="D318" t="str">
+        <v>BL-078 נוסף לבקלוג — UX: תיקון הודעת "מצריכה מובייל" המטעה במדפדפן מובייל לייבוא אנשי קשר ממכשיר; עדיפות 🟢 נמוכה; לא יושם בספרינט הנוכחי</v>
+      </c>
+      <c r="E318" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F318" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G318" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H318" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H317"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H318"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(backlog): add BL-079 — Language/Religion dropdowns in CSV import template
Medium priority improvement: Excel dropdown validation for Language and Religion fields
to prevent spelling errors and inconsistent data on contact import.
No implementation — backlog only.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H318"/>
+  <dimension ref="A1:H319"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8434,9 +8434,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B319" t="str">
+        <v>23:00</v>
+      </c>
+      <c r="C319" t="str">
+        <v>BACKLOG.md / BACKLOG.csv</v>
+      </c>
+      <c r="D319" t="str">
+        <v>BL-079 נוסף לבקלוג — שיפור: הוספת תפריט בחירה של שפה ודת לתבנית ייבוא Excel/CSV; עדיפות 🟡 בינונית; לא יושם בספרינט הנוכחי</v>
+      </c>
+      <c r="E319" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F319" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G319" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H319" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H318"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H319"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(backlog): add BL-080 — incorrect notification timing for Israeli holidays
High priority bug: Yom HaZikaron / Yom HaAtzmaut notifications fired on wrong date.
Suspected: missing Israel mode in Hebcal call or wrong timezone (Asia/Jerusalem).
No implementation — backlog only. BUG-082 logged as open in BUG_REPORT.md.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H323"/>
+  <dimension ref="A1:H324"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8564,9 +8564,35 @@
         <v>done</v>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B324" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C324" t="str">
+        <v>BACKLOG.md / BACKLOG.csv</v>
+      </c>
+      <c r="D324" t="str">
+        <v>BL-080 נוסף לבקלוג — BUG: תזמון שגוי של התראות לחגים ישראליים (יום הזיכרון / יום העצמאות); עדיפות 🔴 גבוהה; לא יושם — ממתין לספרינט מאושר</v>
+      </c>
+      <c r="E324" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F324" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G324" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H324" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H323"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H324"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint18): RTL icons fix, contact card overflow menu, BottomNav active indicator
BL-081: Fix 3 hardcoded ArrowRight icons in ImportContactsScreen — now lang-conditional (ArrowLeft in Hebrew)
BL-075: Add 3-dot overflow menu to ContactCard with Edit/Delete, outside-click/Escape close, delete confirmation modal
BL-049: BottomNav active tab gets inset top border (box-shadow) + stronger glow (opacity-20) for clear distinction
Backlog: Add BL-082 (points system explanation), expand BL-079 (Language-Religion drilldown + single source of truth)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H325"/>
+  <dimension ref="A1:H335"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8616,9 +8616,269 @@
         <v>done</v>
       </c>
     </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B326" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C326" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D326" t="str">
+        <v>BL-081 נוסף לבאקלוג — באג: אייקוני כיוון (ArrowRight) ב-ImportContactsScreen.tsx לא מודעים ל-RTL; 3 מופעים בשורות 188, 292, 334; כל שאר המסכים כבר נכונים</v>
+      </c>
+      <c r="E326" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F326" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G326" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H326" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B327" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C327" t="str">
+        <v>BACKLOG.csv</v>
+      </c>
+      <c r="D327" t="str">
+        <v>BL-081 נוסף ל-BACKLOG.csv עם עדיפות High</v>
+      </c>
+      <c r="E327" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F327" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G327" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H327" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B328" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C328" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D328" t="str">
+        <v>BL-081 תוקן — 3 מופעי ArrowRight קשוחים הוחלפו ב-lang==='he' ? ArrowLeft : ArrowRight; נוסף useLang() ו-ArrowLeft לייבואים; כפתור ייבוא ממכשיר, הורד תבנית, עמודת מיפוי — כולם RTL-נכון</v>
+      </c>
+      <c r="E328" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F328" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G328" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H328" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B329" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C329" t="str">
+        <v>src/components/ContactCard.tsx</v>
+      </c>
+      <c r="D329" t="str">
+        <v>BL-075 יושם — ContactCard קיבל 3-dot overflow menu (MoreVertical); לחיצה פותחת תפריט עם עריכה + מחיקה; מחיקה פותחת Modal אישור; סגירה על-ידי outside click + Escape; aria-label contacts_moreOptions; dropdown מיוצב RTL-aware</v>
+      </c>
+      <c r="E329" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F329" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G329" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H329" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B330" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C330" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D330" t="str">
+        <v>BL-075 — נוסף מפתח contacts_moreOptions ('More options' / 'אפשרויות נוספות') לשני הלוקאלים</v>
+      </c>
+      <c r="E330" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F330" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G330" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H330" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B331" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C331" t="str">
+        <v>src/index.css</v>
+      </c>
+      <c r="D331" t="str">
+        <v>BL-049 — .bottom-nav-item.active קיבל box-shadow: inset 0 2px 0 var(--color-primary); מוסיף פס אינדיקטור עליון ברור לטאב הפעיל</v>
+      </c>
+      <c r="E331" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F331" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G331" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H331" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B332" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C332" t="str">
+        <v>src/components/Navigation.tsx</v>
+      </c>
+      <c r="D332" t="str">
+        <v>BL-049 — גלו רקע לאייקון הפעיל שודרג מ-opacity-15 ל-opacity-20 לניגודיות גבוהה יותר</v>
+      </c>
+      <c r="E332" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F332" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G332" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H332" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B333" t="str">
+        <v>12:35</v>
+      </c>
+      <c r="C333" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D333" t="str">
+        <v>BL-082 נוסף לבאקלוג — שיפור: מערכת הנקודות לא מוסברת; calculateRelationshipScore() ב-scoringSystem.ts; דרוש הסבר UX בעברית ואנגלית</v>
+      </c>
+      <c r="E333" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F333" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G333" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H333" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B334" t="str">
+        <v>12:35</v>
+      </c>
+      <c r="C334" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D334" t="str">
+        <v>BL-079 הורחב — כולל כעת drilldown בין Language ל-Religion ב-UI dropdowns ומקור אחד של אמת (shared config) בנוסף לתבנית ה-CSV</v>
+      </c>
+      <c r="E334" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F334" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G334" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H334" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B335" t="str">
+        <v>12:35</v>
+      </c>
+      <c r="C335" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Sprint 18 סגור — BL-081/BL-075/BL-049 עודכנו ל-Done</v>
+      </c>
+      <c r="E335" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F335" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G335" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H335" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H325"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H335"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint19): Language-Religion drilldown + CSV localization (BL-079)
Add src/data/contactConfig.ts — single source of truth:
- LANGUAGE_KEYS, RELIGION_KEYS canonical arrays
- LANGUAGE_RELIGION_ORDER: Religion options ordered by relevance per contact language
- normalizeLanguage()/normalizeReligion(): accept raw key, EN label, or HE label
- getLanguageDisplayValue()/getReligionDisplayValue(): clean locale-aware display strings

importService.ts: replace direct Language/Religion casts with normalizeLanguage/normalizeReligion
ImportContactsScreen.tsx: CSV template headers and example row now localized per app language
ContactFormScreen.tsx: Religion dropdown reorders options based on selected contact language

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H335"/>
+  <dimension ref="A1:H340"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -8876,9 +8876,139 @@
         <v>done</v>
       </c>
     </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B336" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C336" t="str">
+        <v>src/data/contactConfig.ts</v>
+      </c>
+      <c r="D336" t="str">
+        <v>BL-079 — קובץ config חדש: LANGUAGE_KEYS, RELIGION_KEYS, LANGUAGE_RELIGION_ORDER (drilldown per language), LANGUAGE_DISPLAY + RELIGION_DISPLAY (EN+HE), normalizeLanguage(), normalizeReligion(), getLanguageDisplayValue(), getReligionDisplayValue() — מקור יחיד של אמת</v>
+      </c>
+      <c r="E336" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F336" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G336" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H336" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B337" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C337" t="str">
+        <v>src/services/importService.ts</v>
+      </c>
+      <c r="D337" t="str">
+        <v>BL-079 — הוחלפו cast ישיר (as Language / as Religion) ב-normalizeLanguage() ו-normalizeReligion() מ-contactConfig; מקבל raw key, EN label, ו-HE label</v>
+      </c>
+      <c r="E337" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F337" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G337" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H337" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B338" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C338" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D338" t="str">
+        <v>BL-079 — downloadCSVTemplate() מקבל locale param; headers ו-example row מלוקלים לפי שפת האפליקציה (EN: Name/Phone/Religion=Judaism/Language=English, HE: שם/טלפון/דת=יהדות/שפה=עברית)</v>
+      </c>
+      <c r="E338" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F338" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G338" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H338" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B339" t="str">
+        <v>13:30</v>
+      </c>
+      <c r="C339" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D339" t="str">
+        <v>BL-079 — RELIGION_LABELS מוחלף ב-LANGUAGE_RELIGION_ORDER מ-contactConfig; Religion dropdown מסדר אפשרויות לפי רלוונטיות לשפת הקשר (כל הדתות זמינות, רק סדר שונה)</v>
+      </c>
+      <c r="E339" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F339" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G339" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H339" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B340" t="str">
+        <v>13:35</v>
+      </c>
+      <c r="C340" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D340" t="str">
+        <v>BL-079 עודכן ל-Done Sprint 19</v>
+      </c>
+      <c r="E340" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F340" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G340" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H340" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H335"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H340"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint20): Hebrew Birthday CSV round-trip — import template + parser (BL-076)
- ImportContactsScreen: added 'Hebrew Birthday (DD-MM)' / 'יום הולדת עברי (יום-חודש)' column to downloadCSVTemplate (EN + HE); example row shows '14-07'
- importService: added hebrewBirthday to DETECTABLE_FIELDS (ordered before birthday to prevent false match on 'hebrew birthday' substring); processImport now writes hebrewBirthday to Contact object
- Closes broken export↔import round-trip: exportService already output the column; import now reads it back correctly

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H340"/>
+  <dimension ref="A1:H343"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -9006,9 +9006,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B341" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C341" t="str">
+        <v>src/services/importService.ts</v>
+      </c>
+      <c r="D341" t="str">
+        <v>BL-076 — נוסף hebrewBirthday ל-DETECTABLE_FIELDS (לפני birthday כדי למנוע התאמה שגויה); processImport כותב hebrewBirthday לאובייקט Contact</v>
+      </c>
+      <c r="E341" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F341" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G341" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H341" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B342" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C342" t="str">
+        <v>src/screens/premium/ImportContactsScreen.tsx</v>
+      </c>
+      <c r="D342" t="str">
+        <v>BL-076 — נוסף עמודת 'Hebrew Birthday (DD-MM)' / 'יום הולדת עברי (יום-חודש)' לתבנית CSV להורדה; שורת הדוגמה מציגה 14-07 כדוגמת פורמט</v>
+      </c>
+      <c r="E342" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F342" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G342" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H342" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B343" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C343" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D343" t="str">
+        <v>BL-076 עודכן ל-Done Sprint 20</v>
+      </c>
+      <c r="E343" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F343" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G343" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H343" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H340"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H343"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint21): BL-084 birthday crash fix + BL-082 score tooltip + BL-068/069 group assignment
BL-084 (bug): normalizeBirthday() in importService.ts converts CSV dates to ISO; isNaN guard
in ContactDetailScreen prevents RangeError crash on invalid birthday strings.

BL-082 (improvement): score badge in ContactCard is now a tappable button showing a tooltip
(score_tipTitle + score_tipBody) explaining how the score is calculated. EN+HE. click-outside
and Escape close the tooltip.

BL-068 (feature): contact picker added to GroupsScreen create/edit modal — searchable list
with checkboxes; selectedContactIds initialized from group.contactIds; saved on submit. EN+HE.

BL-069 (feature): optional group selector in ContactFormScreen for new contacts only; after
addContact, calls updateGroup to append the new contact id. EN+HE.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H343"/>
+  <dimension ref="A1:H351"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -9084,9 +9084,217 @@
         <v>done</v>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B344" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C344" t="str">
+        <v>src/services/importService.ts</v>
+      </c>
+      <c r="D344" t="str">
+        <v>BL-084 / BUG-084 — נוסף normalizeBirthday() שמנרמלת תאריכים לפורמט YYYY-MM-DD; מונע שגיאת RangeError כאשר תאריך ה-CSV אינו בפורמט ISO</v>
+      </c>
+      <c r="E344" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F344" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G344" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H344" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B345" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C345" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D345" t="str">
+        <v>BL-084 / BUG-084 — נוסף !isNaN guard לפני format(new Date(contact.birthday)) כדי למנוע קריסה על תאריכים שגויים בנתונים קיימים</v>
+      </c>
+      <c r="E345" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F345" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G345" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H345" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B346" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C346" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D346" t="str">
+        <v>BL-082 — נוספו מפתחות score_tipTitle ו-score_tipBody ב-EN וב-HE לתיאור ציון הקשר</v>
+      </c>
+      <c r="E346" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F346" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G346" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H346" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B347" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C347" t="str">
+        <v>src/components/ContactCard.tsx</v>
+      </c>
+      <c r="D347" t="str">
+        <v>BL-082 — הפיכת תג הציון ל-button ניתן ללחיצה; הוסף tooltip עם הסבר על חישוב הציון; showScoreTip state + click-outside handler</v>
+      </c>
+      <c r="E347" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F347" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G347" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H347" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B348" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C348" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D348" t="str">
+        <v>BL-068 — נוספו מפתחות groups_membersSection, groups_searchContacts, groups_membersSelected ב-EN וב-HE</v>
+      </c>
+      <c r="E348" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F348" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G348" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H348" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B349" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C349" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D349" t="str">
+        <v>BL-068 — נוסף contact picker ב-modal יצירת/עריכת קבוצה; selectedContactIds state; openForm מאתחל מ-group.contactIds; handleSave שומר contactIds</v>
+      </c>
+      <c r="E349" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F349" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G349" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H349" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B350" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C350" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D350" t="str">
+        <v>BL-069 — נוספו מפתחות contactForm_assignGroup ו-contactForm_noGroup ב-EN וב-HE</v>
+      </c>
+      <c r="E350" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F350" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G350" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H350" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B351" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C351" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D351" t="str">
+        <v>BL-069 — נוסף group selector ב-form (מוצג רק לאנשי קשר חדשים); לאחר addContact מעדכן group.contactIds אם נבחרה קבוצה</v>
+      </c>
+      <c r="E351" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F351" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G351" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H351" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H343"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H351"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint22): CSV round-trip data integrity — celebrationType, hebrewBirthday, export warning
BL-092: celebrationType added to DETECTABLE_FIELDS; normalizeCelebrationType() maps
common inputs (Jewish/Christian/Muslim/Druze/Secular); processImport writes field to
Contact. Export↔import round-trip now preserves celebration type.

BL-090: normalizeHebrewBirthday() in importService rejects non-DD-MM strings before
storing. Regex guard in ContactDetailScreen prevents rendering malformed values.

BL-091: settings_exportGroupWarning i18n key (EN+HE); warning note rendered below
CSV export button in SettingsScreen.

Docs: BL-050 and BL-052 corrected to Done (implemented Sprint 5, never updated).
New backlog items BL-086–BL-093 added from gap analysis.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H351"/>
+  <dimension ref="A1:H357"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -9292,9 +9292,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B352" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C352" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D352" t="str">
+        <v>BL-050 ו-BL-052 עודכנו ל-Done — שניהם יושמו בעבר (Sprint 5) אך נשארו בטעות ב-Backlog</v>
+      </c>
+      <c r="E352" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F352" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G352" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H352" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B353" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C353" t="str">
+        <v>src/services/importService.ts</v>
+      </c>
+      <c r="D353" t="str">
+        <v>BL-092 — נוסף celebrationType ל-DETECTABLE_FIELDS; normalizeCelebrationType() ממפה ערכים (Jewish/Christian/Muslim/Druze/Secular); processImport כותב celebrationType לאיש הקשר</v>
+      </c>
+      <c r="E353" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F353" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G353" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H353" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B354" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C354" t="str">
+        <v>src/services/importService.ts</v>
+      </c>
+      <c r="D354" t="str">
+        <v>BL-090 — נוסף normalizeHebrewBirthday() שמאמת פורמט DD-MM; processImport עכשיו מנרמל hebrewBirthday לפני שמירה; ערכים לא תקינים מוחזרים כ-undefined</v>
+      </c>
+      <c r="E354" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F354" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G354" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H354" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B355" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C355" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D355" t="str">
+        <v>BL-090 — נוסף regex guard /^\d{1,2}-\d{1,2}$/ לפני הצגת hebrewBirthday; מונע הצגת שורה ריקה על ערכים לא תקינים</v>
+      </c>
+      <c r="E355" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F355" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G355" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H355" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B356" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C356" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D356" t="str">
+        <v>BL-091 — נוסף מפתח settings_exportGroupWarning ב-EN וב-HE; מזהיר את המשתמש ששיוך לקבוצות לא נכלל בייצוא CSV</v>
+      </c>
+      <c r="E356" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F356" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G356" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H356" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>2026-05-02</v>
+      </c>
+      <c r="B357" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C357" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D357" t="str">
+        <v>BL-091 — נוסף טקסט אזהרה מתחת לכפתור ייצוא CSV: 'שיוך לקבוצות לא נכלל בייצוא ה-CSV'</v>
+      </c>
+      <c r="E357" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F357" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G357" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H357" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H351"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H357"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(mvp): disable Premium gates for MVP phase
All premium restrictions temporarily disabled — every feature accessible
to all users. PremiumBadge/PremiumFeaturePrompt return null, /upgrade and
/payment redirect to dashboard, media attachment gate removed.
Full Premium logic preserved; revert via TEMP comment search.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H361"/>
+  <dimension ref="A1:H370"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -9552,9 +9552,243 @@
         <v>done</v>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B362" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C362" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Sprint 24 — נוספו מפתחות contactDetail_groups, group_religion_filter ב-EN וב-HE; עודכן group_purpose_hint לטקסט ברור יותר (BL-089, BL-093)</v>
+      </c>
+      <c r="E362" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F362" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G362" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H362" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B363" t="str">
+        <v>10:01</v>
+      </c>
+      <c r="C363" t="str">
+        <v>src/components/ContactCard.tsx</v>
+      </c>
+      <c r="D363" t="str">
+        <v>BL-089: הוספת chip קבוצת חברות לכרטיס איש הקשר — מציג עד 2 קבוצות עם צבע + אמוג'י; overflow +N; reverse-lookup דרך Group.contactIds</v>
+      </c>
+      <c r="E363" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F363" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G363" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H363" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B364" t="str">
+        <v>10:02</v>
+      </c>
+      <c r="C364" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D364" t="str">
+        <v>BL-089: נוסף חלק קבוצות במסך פרטי איש קשר — מציג כל הקבוצות שאיש הקשר שייך אליהן; useMemo עם id לפני return מוקדם</v>
+      </c>
+      <c r="E364" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F364" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G364" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H364" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B365" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C365" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D365" t="str">
+        <v>BL-093 Phase 1: נוספו chips סינון לפי דת בחלק הוספת חגים לקבוצה (Premium); מסנן את רשימת החגים לפי הדתות שנבחרו; אין בחירה אוטומטית; מתאפס בפתיחת הטופס</v>
+      </c>
+      <c r="E365" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F365" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G365" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H365" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B366" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C366" t="str">
+        <v>src/context/AppContext.tsx</v>
+      </c>
+      <c r="D366" t="str">
+        <v>TEMP: בוטלו מגבלות פרמיום ל-MVP — canAddContact ו-canAddGroup מוגדרים כ-true ללא תלות ב-isPremium; LIMITS נשמר עם הערת eslint-disable</v>
+      </c>
+      <c r="E366" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F366" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G366" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H366" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B367" t="str">
+        <v>12:01</v>
+      </c>
+      <c r="C367" t="str">
+        <v>src/components/PremiumBadge.tsx</v>
+      </c>
+      <c r="D367" t="str">
+        <v>TEMP: PremiumBadge ו-PremiumFeaturePrompt מחזירים null כשshowPremiumUI=false — הסתרת כל תגיות ו-prompts פרמיום ב-MVP</v>
+      </c>
+      <c r="E367" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F367" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G367" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H367" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B368" t="str">
+        <v>12:02</v>
+      </c>
+      <c r="C368" t="str">
+        <v>src/screens/UpgradeScreen.tsx</v>
+      </c>
+      <c r="D368" t="str">
+        <v>TEMP: מסך Upgrade מפנה ל-/dashboard כשshowPremiumUI=false — מניעת גישה למסך שדרוג ב-MVP</v>
+      </c>
+      <c r="E368" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F368" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G368" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H368" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B369" t="str">
+        <v>12:03</v>
+      </c>
+      <c r="C369" t="str">
+        <v>src/screens/PaymeScreen.tsx</v>
+      </c>
+      <c r="D369" t="str">
+        <v>TEMP: מסך PayMe מפנה ל-/dashboard כשshowPremiumUI=false — מניעת גישה למסך תשלום ב-MVP</v>
+      </c>
+      <c r="E369" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F369" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G369" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H369" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B370" t="str">
+        <v>12:04</v>
+      </c>
+      <c r="C370" t="str">
+        <v>src/components/MediaAttachmentPicker.tsx</v>
+      </c>
+      <c r="D370" t="str">
+        <v>TEMP: שער isPremium ב-MediaAttachmentPicker הוחלף ב-(false as boolean) — צירוף מדיה זמין לכל המשתמשים ב-MVP</v>
+      </c>
+      <c r="E370" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F370" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G370" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H370" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H361"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H370"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint24-25): Group membership chips, holiday language fix, event sort, group edit
Sprint 24 — BL-089/093:
- ContactCard: group chips (up to 2 + overflow)
- ContactDetailScreen: groups section with reverse-lookup
- GroupsScreen: religion filter chips + group purpose copy

Sprint 25 — BL-094/085/096:
- holidayUtils.ts: shared getHolidayDisplayName(holiday, lang) utility
- BL-094: apply getHolidayDisplayName() to all holiday name render points
  (HolidayCard, DashboardScreen, HolidayDetailScreen, HolidayRemindersScreen,
   GreetingEditorScreen, ContactDetailScreen, notificationService, App.tsx,
   GroupsScreen — removes local duplicate)
- BL-085: sort relatedHolidays by date in ContactDetailScreen
- BL-096: group toggle chips + save sync in ContactFormScreen edit mode

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H370"/>
+  <dimension ref="A1:H381"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -9786,9 +9786,295 @@
         <v>done</v>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B371" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C371" t="str">
+        <v>src/utils/holidayUtils.ts</v>
+      </c>
+      <c r="D371" t="str">
+        <v>נוצר util משותף getHolidayDisplayName(holiday, lang) — מחזיר שם חג בשפת הממשק (עברית/אנגלית). BL-094</v>
+      </c>
+      <c r="E371" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F371" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G371" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H371" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B372" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C372" t="str">
+        <v>src/components/HolidayCard.tsx</v>
+      </c>
+      <c r="D372" t="str">
+        <v>BL-094: שם חג מוצג דרך getHolidayDisplayName() — תמיכה בשתי שפות בכרטיס חג</v>
+      </c>
+      <c r="E372" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F372" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G372" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H372" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B373" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C373" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D373" t="str">
+        <v>BL-094: 3 נקודות הצגת שם חג עברו ל-getHolidayDisplayName() — pending item, hero banner, group alert</v>
+      </c>
+      <c r="E373" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F373" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G373" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H373" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B374" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C374" t="str">
+        <v>src/screens/HolidayDetailScreen.tsx</v>
+      </c>
+      <c r="D374" t="str">
+        <v>BL-094: כותרת עמוד וכותרת hero מוצגות דרך getHolidayDisplayName()</v>
+      </c>
+      <c r="E374" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F374" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G374" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H374" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B375" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C375" t="str">
+        <v>src/screens/HolidayRemindersScreen.tsx</v>
+      </c>
+      <c r="D375" t="str">
+        <v>BL-094: שם חג בדף תזכורות חגים מוצג דרך getHolidayDisplayName()</v>
+      </c>
+      <c r="E375" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F375" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G375" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H375" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B376" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C376" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D376" t="str">
+        <v>BL-094: dropdown בחירת חג מציג שם בשפת הממשק דרך getHolidayDisplayName()</v>
+      </c>
+      <c r="E376" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F376" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G376" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H376" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B377" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C377" t="str">
+        <v>src/screens/GroupsScreen.tsx</v>
+      </c>
+      <c r="D377" t="str">
+        <v>BL-094: הוסר duplicate מקומי של getHolidayDisplayName; מייבא עכשיו מ-holidayUtils</v>
+      </c>
+      <c r="E377" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F377" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G377" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H377" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B378" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C378" t="str">
+        <v>src/screens/ContactDetailScreen.tsx</v>
+      </c>
+      <c r="D378" t="str">
+        <v>BL-094: שם חג בפעולת שליחת ברכה מוצג דרך getHolidayDisplayName(). BL-085: חגים קשורים ממוינים לפי תאריך</v>
+      </c>
+      <c r="E378" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F378" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G378" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H378" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B379" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C379" t="str">
+        <v>src/services/notificationService.ts</v>
+      </c>
+      <c r="D379" t="str">
+        <v>BL-094: שמות חגים בהתראות מוצגים בשפת המשתמש — פרמטר lang נוסף ל-fireReminders()</v>
+      </c>
+      <c r="E379" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F379" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G379" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H379" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B380" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C380" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="D380" t="str">
+        <v>BL-094: lang מ-useLang() מועבר ל-fireReminders() לתמיכה בהתראות בשפת המשתמש</v>
+      </c>
+      <c r="E380" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F380" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G380" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H380" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B381" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C381" t="str">
+        <v>src/screens/ContactFormScreen.tsx</v>
+      </c>
+      <c r="D381" t="str">
+        <v>BL-096: נוספה אפשרות לשיוך/הסרה מקבוצות בעריכת איש קשר קיים — chips toggle UI + סנכרון בשמירה</v>
+      </c>
+      <c r="E381" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F381" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G381" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H381" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H370"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H381"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint26): Empty state UX + QuickAddModal — first contact in under 30s (BL-098/099)
BL-098: Dashboard and ContactsScreen empty states updated with emotionally
resonant messaging ("Who matters to you?" / "מי חשוב לך?"). CTA now opens
QuickAddModal instead of navigating to the full 10-field form.

BL-099: New QuickAddModal bottom sheet — name + phone required, all other
fields set to defaults. State resets cleanly on each open via conditional
mount. Link to full form available for users who want to add more details.
FAB and header Add button still navigate to full ContactFormScreen.

Both EN and HE locales updated. 8 new quickAdd_* i18n keys added.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H381"/>
+  <dimension ref="A1:H387"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -10072,9 +10072,165 @@
         <v>done</v>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="B382" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C382" t="str">
+        <v>src/components/QuickAddModal.tsx</v>
+      </c>
+      <c r="D382" t="str">
+        <v>BL-099: נוצר QuickAddModal — bottom sheet עם שדות שם + טלפון בלבד; שמירה יוצרת איש קשר עם ברירות מחדל; סגירה לאחר שמירה; קישור לטופס מלא</v>
+      </c>
+      <c r="E382" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F382" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G382" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H382" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="B383" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C383" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D383" t="str">
+        <v>BL-098/099: עדכון מחרוזות empty state לניסוח רגשי/ערכי (EN+HE); נוספו 8 מפתחות quickAdd_* (title, name, phone, placeholders, save, required, fullForm) — EN+HE</v>
+      </c>
+      <c r="E383" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F383" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G383" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H383" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="B384" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C384" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D384" t="str">
+        <v>BL-098/099: empty state ב-Dashboard משתמש ב-QuickAddModal במקום ניווט לטופס מלא; אייקון 💛; CTA מוביל להוספה מהירה</v>
+      </c>
+      <c r="E384" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F384" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G384" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H384" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="B385" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C385" t="str">
+        <v>src/screens/ContactsScreen.tsx</v>
+      </c>
+      <c r="D385" t="str">
+        <v>BL-098/099: empty state ב-ContactsScreen משתמש ב-QuickAddModal במקום ניווט לטופס מלא; FAB ממשיך לנווט לטופס מלא</v>
+      </c>
+      <c r="E385" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F385" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G385" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H385" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="B386" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C386" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D386" t="str">
+        <v>BL-098 ו-BL-099 נוספו לבקלוג וסומנו Done — Sprint 26</v>
+      </c>
+      <c r="E386" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F386" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G386" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H386" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>2026-05-05</v>
+      </c>
+      <c r="B387" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C387" t="str">
+        <v>BACKLOG.csv</v>
+      </c>
+      <c r="D387" t="str">
+        <v>BL-098 ו-BL-099 נוספו לבקלוג.csv וסומנו Done — Sprint 26</v>
+      </c>
+      <c r="E387" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F387" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G387" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H387" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H381"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H387"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint27): BL-100 contact dropdown placeholder fix + BL-083 FeatureGuide
BL-100: Select component now supports disabled/hidden on option objects;
GreetingEditorScreen contact placeholder uses disabled+hidden so it is
display-only and cannot be selected.

BL-083: FeatureGuide bottom sheet (3 slides, dot indicators, RTL-aware
back/next, skippable via X). Shown on first launch via DashboardScreen;
re-accessible from Settings > App info > Feature Guide (resets nm_guide_seen).
localStorage helpers extracted to src/utils/featureGuideUtils.ts to satisfy
react-refresh/only-export-components lint rule.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H387"/>
+  <dimension ref="A1:H396"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -10228,9 +10228,243 @@
         <v>done</v>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B388" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C388" t="str">
+        <v>src/components/ui/Select.tsx</v>
+      </c>
+      <c r="D388" t="str">
+        <v>BL-100: הוספת שדות disabled ו-hidden לטיפוס option ב-Select — תומך ב-placeholder שלא ניתן לבחור</v>
+      </c>
+      <c r="E388" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F388" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G388" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H388" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B389" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C389" t="str">
+        <v>src/screens/GreetingEditorScreen.tsx</v>
+      </c>
+      <c r="D389" t="str">
+        <v>BL-100: placeholder 'בחר איש קשר' ב-dropdown ה-contact עם disabled+hidden — לא ניתן לשמור עם placeholder</v>
+      </c>
+      <c r="E389" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F389" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G389" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H389" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B390" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C390" t="str">
+        <v>src/utils/featureGuideUtils.ts</v>
+      </c>
+      <c r="D390" t="str">
+        <v>BL-083: עזרי localStorage לפיצ'ר guide — isGuideSeen, markGuideSeen, resetGuide עם מפתח nm_guide_seen</v>
+      </c>
+      <c r="E390" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F390" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G390" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H390" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B391" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C391" t="str">
+        <v>src/components/FeatureGuide.tsx</v>
+      </c>
+      <c r="D391" t="str">
+        <v>BL-083: קומפוננטת FeatureGuide — 3 שקפים עם אמוג'י, כותרת, גוף; כפתור דלג (X) בכל שקף; מחוונים מנוקדים; ניווט RTL-aware; CTA 'בואו נתחיל'</v>
+      </c>
+      <c r="E391" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F391" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G391" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H391" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B392" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C392" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D392" t="str">
+        <v>BL-083/BL-100: נוספו מפתחות guide_slide1_title/body, guide_slide2_title/body, guide_slide3_title/body, guide_next, guide_done, guide_viewGuide, greeting_selectContact — EN + HE</v>
+      </c>
+      <c r="E392" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F392" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G392" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H392" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B393" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C393" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D393" t="str">
+        <v>BL-083: חיבור FeatureGuide — state showGuide מ-isGuideSeen(); מוצג בעלייה ראשונה לאפליקציה; נסגר ב-onDone</v>
+      </c>
+      <c r="E393" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F393" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G393" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H393" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B394" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C394" t="str">
+        <v>src/screens/SettingsScreen.tsx</v>
+      </c>
+      <c r="D394" t="str">
+        <v>BL-083: כפתור 'Feature Guide' בסעיף App info — מאפס nm_guide_seen ומנווט ל-Dashboard כדי שה-Guide יוצג מחדש</v>
+      </c>
+      <c r="E394" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F394" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G394" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H394" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B395" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C395" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D395" t="str">
+        <v>BL-100 ו-BL-083 סומנו Done — Sprint 27</v>
+      </c>
+      <c r="E395" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F395" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G395" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H395" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>2026-05-04</v>
+      </c>
+      <c r="B396" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C396" t="str">
+        <v>BACKLOG.csv</v>
+      </c>
+      <c r="D396" t="str">
+        <v>BL-100 ו-BL-083 עודכנו ל-Done — Sprint 27</v>
+      </c>
+      <c r="E396" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F396" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G396" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H396" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H387"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H396"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint28): BL-097 Landing page — emotional entry point before app
- LandingScreen: 4 relationship WebP images (Romantic/Family/Friends/work),
  hero tagline, 3 CTAs (Get Started / Log In Coming Soon / Try Demo)
- dontShowLanding localStorage flag via storageService + appConfig
- Root redirect checks dontShowLanding first; returning users auto-skip
- Login CTA shows coming-soon note inline — no fake auth
- Demo reuses existing enableDemo() + markOnboardingDone() unchanged
- 14 i18n keys added EN + HE
- changelog.xlsx 402 entries; QA checklist 166 tests (164 ✅)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H396"/>
+  <dimension ref="A1:H403"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -10462,9 +10462,191 @@
         <v>done</v>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B397" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C397" t="str">
+        <v>src/config/appConfig.ts</v>
+      </c>
+      <c r="D397" t="str">
+        <v>Sprint 28 — BL-097: הוסף מפתח אחסון nm_dont_show_landing ל-storageKeys</v>
+      </c>
+      <c r="E397" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F397" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G397" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H397" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B398" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C398" t="str">
+        <v>src/services/storageService.ts</v>
+      </c>
+      <c r="D398" t="str">
+        <v>Sprint 28 — BL-097: הוסף isDontShowLanding() ו-setDontShowLanding() לניהול דגל דף הנחיתה</v>
+      </c>
+      <c r="E398" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F398" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G398" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H398" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B399" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C399" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D399" t="str">
+        <v>Sprint 28 — BL-097: הוסף 14 מפתחות תרגום לדף הנחיתה — EN ו-HE (tagline, subtitle, CTAs, scene labels, captions)</v>
+      </c>
+      <c r="E399" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F399" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G399" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H399" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B400" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C400" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D400" t="str">
+        <v>Sprint 28 — BL-097: נוצר דף נחיתה — ערך רגשי, 4 תמונות קשרים (זוגיות/משפחה/חברים/עבודה), 3 כפתורי CTA, דגל dontShowLanding, דילוג אוטומטי למשתמש חוזר</v>
+      </c>
+      <c r="E400" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F400" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G400" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H400" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B401" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C401" t="str">
+        <v>src/assets/landing/</v>
+      </c>
+      <c r="D401" t="str">
+        <v>Sprint 28 — BL-097: נוספו 4 תמונות WebP אופטימליות לדף הנחיתה (Romantic/Family/Friends/work)</v>
+      </c>
+      <c r="E401" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F401" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G401" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H401" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B402" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C402" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="D402" t="str">
+        <v>Sprint 28 — BL-097: הוסף נתיב /landing ועדכן redirect שורש לבדיקת dontShowLanding לפני onboarding</v>
+      </c>
+      <c r="E402" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F402" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G402" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H402" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B403" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C403" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Sprint 28 — תוקן lint: הסרת ייבוא isDontShowLanding שלא היה בשימוש ב-LandingScreen</v>
+      </c>
+      <c r="E403" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F403" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G403" t="str">
+        <v>Reviewer</v>
+      </c>
+      <c r="H403" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H396"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H403"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sprint29): Phase 0 backend foundation — AuthContext, dataService, AppContext async-ready
- AuthContext stub (Phase 0): always unauthenticated, async signIn/signOut stubs ready for Phase 1 Supabase
- dataService.ts: async CRUD interface wrapping localStorage; Phase 2 Supabase placeholders in every write
- deleteContactCascade: atomic contact + group membership cleanup
- AppContext refactored: all 9 CRUD mutations route through dataService with fire-and-forget error logging
- Functional state updates throughout (no read-after-write)
- userId? field added to Contact, Group, GreetingDraft (backward-compatible)
- generateId() upgraded to crypto.randomUUID() with fallback
- AuthProvider wired into App.tsx provider tree
- BL-060 marked Done: all required national/secular holidays already in holidays.ts
- QA: 167 tests, 165 ✅

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H403"/>
+  <dimension ref="A1:H410"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -10644,9 +10644,191 @@
         <v>done</v>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B404" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="C404" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D404" t="str">
+        <v>מיקרו-פיקס FINDING-01 — handleRegister ניווט ל-/onboarding בלי לבדוק אם אונבורדינג כבר הושלם; תוקן ל-postLandingDestination() שמנתב למסך הנכון למשתמש חוזר</v>
+      </c>
+      <c r="E404" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F404" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G404" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H404" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B405" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C405" t="str">
+        <v>src/types/index.ts</v>
+      </c>
+      <c r="D405" t="str">
+        <v>ספרינט 29 Phase 0 — הוסף שדה userId?: string אופציונלי ל-Contact, Group, GreetingDraft; מזהה Supabase auth.uid() לשימוש עתידי; תואם לאחור עם נתוני localStorage קיימים</v>
+      </c>
+      <c r="E405" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F405" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G405" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H405" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B406" t="str">
+        <v>10:01</v>
+      </c>
+      <c r="C406" t="str">
+        <v>src/services/storageService.ts</v>
+      </c>
+      <c r="D406" t="str">
+        <v>ספרינט 29 Phase 0 — עדכון generateId() לשימוש ב-crypto.randomUUID() עם fallback לפורמט timestamp ישן; UUID תקני לכל הישויות החדשות</v>
+      </c>
+      <c r="E406" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F406" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G406" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H406" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B407" t="str">
+        <v>10:02</v>
+      </c>
+      <c r="C407" t="str">
+        <v>src/context/AuthContext.tsx</v>
+      </c>
+      <c r="D407" t="str">
+        <v>ספרינט 29 Phase 0 — יצירת AuthContext חדש: stub Phase 0 תמיד לא-מאומת (user: null); מכין את התשתית ל-Supabase magic link auth ב-Phase 1; מייצא AuthUser, AuthProvider, useAuth</v>
+      </c>
+      <c r="E407" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F407" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G407" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H407" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B408" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C408" t="str">
+        <v>src/services/dataService.ts</v>
+      </c>
+      <c r="D408" t="str">
+        <v>ספרינט 29 Phase 0 — יצירת dataService חדש: ממשק async לכל פעולות CRUD (contacts, groups, drafts, settings, premium); Phase 0 = קריאות synchronous ל-localStorage; פקקי Phase 2 ל-Supabase בכל פעולת כתיבה; deleteContactCascade מטפל במחיקה אטומית של איש קשר + ניקוי קבוצות</v>
+      </c>
+      <c r="E408" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F408" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G408" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H408" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B409" t="str">
+        <v>10:04</v>
+      </c>
+      <c r="C409" t="str">
+        <v>src/context/AppContext.tsx</v>
+      </c>
+      <c r="D409" t="str">
+        <v>ספרינט 29 Phase 0 — שידוד AppContext: כל 9 מוטציות CRUD מנותבות דרך dataService עם fire-and-forget; functional state updates (אין read-after-write); auth.user?.id מוצמד לישויות חדשות; useAuth() מיובא; ממשק AppContextValue ציבורי לא שונה — אפס שינויים בסקרינים</v>
+      </c>
+      <c r="E409" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F409" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G409" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H409" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>2026-05-06</v>
+      </c>
+      <c r="B410" t="str">
+        <v>10:05</v>
+      </c>
+      <c r="C410" t="str">
+        <v>src/App.tsx</v>
+      </c>
+      <c r="D410" t="str">
+        <v>ספרינט 29 Phase 0 — הוסף AuthProvider wrapper בין LanguageProvider ל-ThemeProvider; AppProvider כעת רץ בתוך AuthContext</v>
+      </c>
+      <c r="E410" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F410" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G410" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H410" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H403"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H410"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(mobile): prevent auth error layout jump and safe-area clipping on LandingScreen
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H410"/>
+  <dimension ref="A1:H418"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -10826,9 +10826,217 @@
         <v>done</v>
       </c>
     </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B411" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="C411" t="str">
+        <v>src/screens/DashboardScreen.tsx</v>
+      </c>
+      <c r="D411" t="str">
+        <v>BL-113: נוסף sortedUpcomingHolidays useMemo שממיין אירועים עולים לפי תאריך; כל 4 נקודות גישה עודכנו — todayHoliday, tomorrowHoliday, nextHoliday, render slice</v>
+      </c>
+      <c r="E411" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F411" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G411" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H411" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B412" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="C412" t="str">
+        <v>src/context/AppContext.tsx</v>
+      </c>
+      <c r="D412" t="str">
+        <v>BL-112: נוסף useEffect עם מאזין visibilitychange; todayKey state מאלץ חישוב מחדש של dashboardData כשתאריך הלוח השנה משתנה (לאחר חצות); ניקוי listener נעשה ב-cleanup</v>
+      </c>
+      <c r="E412" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F412" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G412" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H412" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B413" t="str">
+        <v>12:20</v>
+      </c>
+      <c r="C413" t="str">
+        <v>src/i18n/index.ts</v>
+      </c>
+      <c r="D413" t="str">
+        <v>BL-122+BL-120: נוספו 3 מפתחות EN+HE — landing_cta_anonymous (המשך בלי חשבון), landing_login_error_rate_limit, landing_login_error_invalid_email</v>
+      </c>
+      <c r="E413" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F413" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G413" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H413" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B414" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C414" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D414" t="str">
+        <v>BL-122: נוספה פונקציה localizeAuthError שממפה שגיאות Supabase גולמיות להודעות עברית ידידותיות למשתמש; לא מוצגות שגיאות אנגלית למשתמשי עברית</v>
+      </c>
+      <c r="E414" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F414" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G414" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H414" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B415" t="str">
+        <v>12:35</v>
+      </c>
+      <c r="C415" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D415" t="str">
+        <v>BL-120: כפתור המשך בלי חשבון (h-12, border) הוחלף במקום קישור אל תציג שוב הזעיר; כפתור ההדגמה הוקטן; נתיב אנונימי הפך לCTA ראשי גלוי מעל הגלילה</v>
+      </c>
+      <c r="E415" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F415" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G415" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H415" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B416" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="C416" t="str">
+        <v>agent_state/changelog_queue.json</v>
+      </c>
+      <c r="D416" t="str">
+        <v>ספרינט 31 — Reviewer אישר: build ✅ lint ✅ RTL ✅ i18n EN+HE ✅ ניקוי listener ✅ אין רגרסיות</v>
+      </c>
+      <c r="E416" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F416" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G416" t="str">
+        <v>Reviewer</v>
+      </c>
+      <c r="H416" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B417" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="C417" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D417" t="str">
+        <v>תוקן BUG-mobile: הודעת שגיאה ב-auth מוצגת בתוך wrapper עם min-h קבוע — מונע קפיצת layout; leading-relaxed + break-words לגלישת שורות בטוחה; red-600 לניגוד טוב יותר</v>
+      </c>
+      <c r="E417" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F417" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G417" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H417" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v>2026-05-08</v>
+      </c>
+      <c r="B418" t="str">
+        <v>21:00</v>
+      </c>
+      <c r="C418" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D418" t="str">
+        <v>תוקן BUG-mobile: bottom spacer עודכן ל-max(2.5rem, env(safe-area-inset-bottom) + 1rem) — כפתור Cancel אינו נחסם על ידי home indicator ב-iPhone X+</v>
+      </c>
+      <c r="E418" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F418" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G418" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H418" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H410"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H418"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BL-133): raise landing screen bottom spacer to clear Android browser chrome
Minimum spacer height increased from max(2.5rem, safe-area+1rem) to
max(5rem, safe-area+2rem). env(safe-area-inset-bottom) is 0 on Android,
so the previous fix did not clear the ~56px Chrome/Samsung Internet
bottom toolbar. 80px floor provides 24px of breathing room above it.
iOS home-indicator path (safe-area-inset-bottom) unchanged.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H418"/>
+  <dimension ref="A1:H421"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -11034,9 +11034,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="B419" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C419" t="str">
+        <v>src/screens/LandingScreen.tsx</v>
+      </c>
+      <c r="D419" t="str">
+        <v>BL-133: spacer תחתון הוגדל מ-max(2.5rem, safe-area+1rem) ל-max(5rem, safe-area+2rem) — מבטיח 80px מינימום כדי לפנות מקום מעל סרגל הניווט של דפדפן Android Chrome ו-Samsung Internet (~56px); אין שינוי ב-iOS</v>
+      </c>
+      <c r="E419" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F419" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G419" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H419" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="B420" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C420" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D420" t="str">
+        <v>BL-133 נוסף לבאקלוג — Mobile browser bottom-bar overlap on landing screen; סטטוס: Done; ספרינט 31 stabilization</v>
+      </c>
+      <c r="E420" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F420" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G420" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H420" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="B421" t="str">
+        <v>00:00</v>
+      </c>
+      <c r="C421" t="str">
+        <v>BACKLOG.csv</v>
+      </c>
+      <c r="D421" t="str">
+        <v>BL-133 נוסף ל-BACKLOG.csv</v>
+      </c>
+      <c r="E421" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F421" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G421" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H421" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H418"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H421"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(BL-134): raise onboarding bottom padding to clear Android browser chrome
Primary CTA (h-14) was partially hidden behind Android Chrome / Samsung
Internet bottom toolbar (~56px). Bottom section used p-6 (24px) with no
safe-area protection. Replace with px-6 pt-6 + paddingBottom
max(5rem, calc(env(safe-area-inset-bottom) + 2rem)). 80px floor clears
the browser bar; flex-1 content area redistributes naturally.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/changelog.xlsx
+++ b/changelog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H421"/>
+  <dimension ref="A1:H424"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="8.83203125" customWidth="1"/>
@@ -11112,9 +11112,87 @@
         <v>done</v>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="B422" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C422" t="str">
+        <v>src/screens/OnboardingScreen.tsx</v>
+      </c>
+      <c r="D422" t="str">
+        <v>BL-134: paddingBottom של bottom section הוגדל מ-p-6 (24px) ל-max(5rem, safe-area+2rem) — כפתור CTA ראשי אינו נחסם על ידי סרגל דפדפן Android Chrome / Samsung Internet</v>
+      </c>
+      <c r="E422" t="str">
+        <v>bugfix</v>
+      </c>
+      <c r="F422" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G422" t="str">
+        <v>Developer</v>
+      </c>
+      <c r="H422" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="B423" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C423" t="str">
+        <v>BACKLOG.md</v>
+      </c>
+      <c r="D423" t="str">
+        <v>BL-134 נוסף לבאקלוג — Onboarding screen CTA hidden behind Android browser chrome; סטטוס: Done</v>
+      </c>
+      <c r="E423" t="str">
+        <v>feature</v>
+      </c>
+      <c r="F423" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G423" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H423" t="str">
+        <v>done</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="B424" t="str">
+        <v>01:00</v>
+      </c>
+      <c r="C424" t="str">
+        <v>BACKLOG.csv</v>
+      </c>
+      <c r="D424" t="str">
+        <v>BL-134 נוסף ל-BACKLOG.csv</v>
+      </c>
+      <c r="E424" t="str">
+        <v>improvement</v>
+      </c>
+      <c r="F424" t="str">
+        <v>code_change</v>
+      </c>
+      <c r="G424" t="str">
+        <v>Documentation</v>
+      </c>
+      <c r="H424" t="str">
+        <v>done</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H421"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H424"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>